<commit_message>
MIA: run automatico 2026-10-30 22:27 UTC
</commit_message>
<xml_diff>
--- a/database/ASAI3.xlsx
+++ b/database/ASAI3.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1417"/>
+  <dimension ref="A1:F1418"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -452,16 +452,16 @@
         <v>44256</v>
       </c>
       <c r="B2" t="n">
-        <v>13.55914783477783</v>
+        <v>13.55914878845215</v>
       </c>
       <c r="C2" t="n">
-        <v>14.43840408118833</v>
+        <v>14.43840509670459</v>
       </c>
       <c r="D2" t="n">
-        <v>13.17554232187502</v>
+        <v>13.17554324856868</v>
       </c>
       <c r="E2" t="n">
-        <v>13.67498995526467</v>
+        <v>13.67499091708668</v>
       </c>
       <c r="F2" t="n">
         <v>64088000</v>
@@ -472,16 +472,16 @@
         <v>44257</v>
       </c>
       <c r="B3" t="n">
-        <v>13.76804351806641</v>
+        <v>13.76804447174072</v>
       </c>
       <c r="C3" t="n">
-        <v>14.0528997719606</v>
+        <v>14.05290074536612</v>
       </c>
       <c r="D3" t="n">
-        <v>13.00462933717113</v>
+        <v>13.00463023796586</v>
       </c>
       <c r="E3" t="n">
-        <v>13.37114384656537</v>
+        <v>13.37114477274755</v>
       </c>
       <c r="F3" t="n">
         <v>14717000</v>
@@ -512,16 +512,16 @@
         <v>44259</v>
       </c>
       <c r="B5" t="n">
-        <v>13.90097618103027</v>
+        <v>13.90097522735596</v>
       </c>
       <c r="C5" t="n">
-        <v>14.04340385011868</v>
+        <v>14.04340288667314</v>
       </c>
       <c r="D5" t="n">
-        <v>13.44330710721157</v>
+        <v>13.44330618493557</v>
       </c>
       <c r="E5" t="n">
-        <v>13.53256187643049</v>
+        <v>13.53256094803118</v>
       </c>
       <c r="F5" t="n">
         <v>12300000</v>
@@ -552,16 +552,16 @@
         <v>44263</v>
       </c>
       <c r="B7" t="n">
-        <v>13.48508644104004</v>
+        <v>13.48508739471436</v>
       </c>
       <c r="C7" t="n">
-        <v>14.2978757345337</v>
+        <v>14.29787674568901</v>
       </c>
       <c r="D7" t="n">
-        <v>13.05210579563423</v>
+        <v>13.05210671868786</v>
       </c>
       <c r="E7" t="n">
-        <v>14.21051986319279</v>
+        <v>14.21052086817024</v>
       </c>
       <c r="F7" t="n">
         <v>12366000</v>
@@ -572,16 +572,16 @@
         <v>44264</v>
       </c>
       <c r="B8" t="n">
-        <v>13.44520568847656</v>
+        <v>13.4452075958252</v>
       </c>
       <c r="C8" t="n">
-        <v>13.44520568847656</v>
+        <v>13.4452075958252</v>
       </c>
       <c r="D8" t="n">
-        <v>13.0103252694391</v>
+        <v>13.01032711509522</v>
       </c>
       <c r="E8" t="n">
-        <v>13.29138370087542</v>
+        <v>13.29138558640273</v>
       </c>
       <c r="F8" t="n">
         <v>10167000</v>
@@ -612,16 +612,16 @@
         <v>44266</v>
       </c>
       <c r="B10" t="n">
-        <v>13.95604801177979</v>
+        <v>13.95604705810547</v>
       </c>
       <c r="C10" t="n">
-        <v>14.15544729222492</v>
+        <v>14.15544632492482</v>
       </c>
       <c r="D10" t="n">
-        <v>13.63510989807421</v>
+        <v>13.63510896633091</v>
       </c>
       <c r="E10" t="n">
-        <v>13.71297125079192</v>
+        <v>13.71297031372804</v>
       </c>
       <c r="F10" t="n">
         <v>16646000</v>
@@ -632,16 +632,16 @@
         <v>44267</v>
       </c>
       <c r="B11" t="n">
-        <v>13.82121658325195</v>
+        <v>13.82121562957764</v>
       </c>
       <c r="C11" t="n">
-        <v>14.06049554958161</v>
+        <v>14.06049457939686</v>
       </c>
       <c r="D11" t="n">
-        <v>13.57813981118895</v>
+        <v>13.57813887428711</v>
       </c>
       <c r="E11" t="n">
-        <v>13.57813981118895</v>
+        <v>13.57813887428711</v>
       </c>
       <c r="F11" t="n">
         <v>7509000</v>
@@ -652,16 +652,16 @@
         <v>44270</v>
       </c>
       <c r="B12" t="n">
-        <v>13.83450984954834</v>
+        <v>13.83450889587402</v>
       </c>
       <c r="C12" t="n">
-        <v>14.01681810828169</v>
+        <v>14.01681714204006</v>
       </c>
       <c r="D12" t="n">
-        <v>13.62181733379263</v>
+        <v>13.62181639478016</v>
       </c>
       <c r="E12" t="n">
-        <v>13.81931772103716</v>
+        <v>13.81931676841011</v>
       </c>
       <c r="F12" t="n">
         <v>11593000</v>
@@ -672,16 +672,16 @@
         <v>44271</v>
       </c>
       <c r="B13" t="n">
-        <v>13.58763408660889</v>
+        <v>13.5876350402832</v>
       </c>
       <c r="C13" t="n">
-        <v>13.91047018507921</v>
+        <v>13.9104711614124</v>
       </c>
       <c r="D13" t="n">
-        <v>13.49458060971476</v>
+        <v>13.49458155685794</v>
       </c>
       <c r="E13" t="n">
-        <v>13.84400406267841</v>
+        <v>13.84400503434655</v>
       </c>
       <c r="F13" t="n">
         <v>7789500</v>
@@ -692,16 +692,16 @@
         <v>44272</v>
       </c>
       <c r="B14" t="n">
-        <v>14.05290031433105</v>
+        <v>14.05289840698242</v>
       </c>
       <c r="C14" t="n">
-        <v>14.07189024903928</v>
+        <v>14.07188833911321</v>
       </c>
       <c r="D14" t="n">
-        <v>13.49458210759284</v>
+        <v>13.49458027602269</v>
       </c>
       <c r="E14" t="n">
-        <v>13.58763559481576</v>
+        <v>13.5876337506158</v>
       </c>
       <c r="F14" t="n">
         <v>4753000</v>
@@ -712,16 +712,16 @@
         <v>44273</v>
       </c>
       <c r="B15" t="n">
-        <v>13.91047191619873</v>
+        <v>13.91047096252441</v>
       </c>
       <c r="C15" t="n">
-        <v>14.01302082492147</v>
+        <v>14.0130198642166</v>
       </c>
       <c r="D15" t="n">
-        <v>13.69018378074197</v>
+        <v>13.69018284217017</v>
       </c>
       <c r="E15" t="n">
-        <v>13.69018378074197</v>
+        <v>13.69018284217017</v>
       </c>
       <c r="F15" t="n">
         <v>2304000</v>
@@ -752,16 +752,16 @@
         <v>44277</v>
       </c>
       <c r="B17" t="n">
-        <v>13.29328346252441</v>
+        <v>13.2932825088501</v>
       </c>
       <c r="C17" t="n">
-        <v>13.63511042556885</v>
+        <v>13.6351094473715</v>
       </c>
       <c r="D17" t="n">
-        <v>13.15655249620002</v>
+        <v>13.15655155233494</v>
       </c>
       <c r="E17" t="n">
-        <v>13.63511042556885</v>
+        <v>13.6351094473715</v>
       </c>
       <c r="F17" t="n">
         <v>5803000</v>
@@ -792,16 +792,16 @@
         <v>44279</v>
       </c>
       <c r="B19" t="n">
-        <v>13.00842666625977</v>
+        <v>13.00842761993408</v>
       </c>
       <c r="C19" t="n">
-        <v>13.4717924479973</v>
+        <v>13.4717934356419</v>
       </c>
       <c r="D19" t="n">
-        <v>12.86599899729744</v>
+        <v>12.86599994053009</v>
       </c>
       <c r="E19" t="n">
-        <v>13.31417265130471</v>
+        <v>13.31417362739389</v>
       </c>
       <c r="F19" t="n">
         <v>12174500</v>
@@ -892,16 +892,16 @@
         <v>44286</v>
       </c>
       <c r="B24" t="n">
-        <v>14.02251529693604</v>
+        <v>14.0225133895874</v>
       </c>
       <c r="C24" t="n">
-        <v>14.04150613737493</v>
+        <v>14.04150422744316</v>
       </c>
       <c r="D24" t="n">
-        <v>13.67499161002203</v>
+        <v>13.67498974994372</v>
       </c>
       <c r="E24" t="n">
-        <v>13.96744348962283</v>
+        <v>13.96744158976508</v>
       </c>
       <c r="F24" t="n">
         <v>3663000</v>
@@ -932,16 +932,16 @@
         <v>44291</v>
       </c>
       <c r="B26" t="n">
-        <v>14.71756362915039</v>
+        <v>14.71756458282471</v>
       </c>
       <c r="C26" t="n">
-        <v>14.88657865823869</v>
+        <v>14.88657962286491</v>
       </c>
       <c r="D26" t="n">
-        <v>14.29977512456389</v>
+        <v>14.29977605116619</v>
       </c>
       <c r="E26" t="n">
-        <v>14.29977512456389</v>
+        <v>14.29977605116619</v>
       </c>
       <c r="F26" t="n">
         <v>6073500</v>
@@ -972,16 +972,16 @@
         <v>44293</v>
       </c>
       <c r="B28" t="n">
-        <v>14.4934778213501</v>
+        <v>14.49347686767578</v>
       </c>
       <c r="C28" t="n">
-        <v>14.78023299581345</v>
+        <v>14.78023202327058</v>
       </c>
       <c r="D28" t="n">
-        <v>13.92756398980291</v>
+        <v>13.92756307336586</v>
       </c>
       <c r="E28" t="n">
-        <v>14.45359814255714</v>
+        <v>14.45359719150692</v>
       </c>
       <c r="F28" t="n">
         <v>10992000</v>
@@ -1012,16 +1012,16 @@
         <v>44295</v>
       </c>
       <c r="B30" t="n">
-        <v>14.71756362915039</v>
+        <v>14.71756458282471</v>
       </c>
       <c r="C30" t="n">
-        <v>14.73655446848903</v>
+        <v>14.73655542339393</v>
       </c>
       <c r="D30" t="n">
-        <v>14.40801982998176</v>
+        <v>14.40802076359814</v>
       </c>
       <c r="E30" t="n">
-        <v>14.63210666319261</v>
+        <v>14.63210761132946</v>
       </c>
       <c r="F30" t="n">
         <v>7012500</v>
@@ -1032,16 +1032,16 @@
         <v>44298</v>
       </c>
       <c r="B31" t="n">
-        <v>14.69857215881348</v>
+        <v>14.69857311248779</v>
       </c>
       <c r="C31" t="n">
-        <v>14.8011210568803</v>
+        <v>14.8011220172082</v>
       </c>
       <c r="D31" t="n">
-        <v>14.52765913976815</v>
+        <v>14.52766008235327</v>
       </c>
       <c r="E31" t="n">
-        <v>14.69857215881348</v>
+        <v>14.69857311248779</v>
       </c>
       <c r="F31" t="n">
         <v>4711000</v>
@@ -1132,16 +1132,16 @@
         <v>44305</v>
       </c>
       <c r="B36" t="n">
-        <v>15.28727531433105</v>
+        <v>15.28727436065674</v>
       </c>
       <c r="C36" t="n">
-        <v>15.50756433010704</v>
+        <v>15.50756336269031</v>
       </c>
       <c r="D36" t="n">
-        <v>15.00431798094175</v>
+        <v>15.00431704491931</v>
       </c>
       <c r="E36" t="n">
-        <v>15.14484674350704</v>
+        <v>15.14484579871793</v>
       </c>
       <c r="F36" t="n">
         <v>5017000</v>
@@ -1152,16 +1152,16 @@
         <v>44306</v>
       </c>
       <c r="B37" t="n">
-        <v>15.47718143463135</v>
+        <v>15.47718048095703</v>
       </c>
       <c r="C37" t="n">
-        <v>15.65569281594117</v>
+        <v>15.65569185126732</v>
       </c>
       <c r="D37" t="n">
-        <v>15.06698938480104</v>
+        <v>15.06698845640197</v>
       </c>
       <c r="E37" t="n">
-        <v>15.35944219725644</v>
+        <v>15.35944125083699</v>
       </c>
       <c r="F37" t="n">
         <v>6029000</v>
@@ -1192,16 +1192,16 @@
         <v>44309</v>
       </c>
       <c r="B39" t="n">
-        <v>15.41261291503906</v>
+        <v>15.41261386871338</v>
       </c>
       <c r="C39" t="n">
-        <v>15.53794955811708</v>
+        <v>15.53795051954675</v>
       </c>
       <c r="D39" t="n">
-        <v>15.218910336355</v>
+        <v>15.21891127804373</v>
       </c>
       <c r="E39" t="n">
-        <v>15.45819020544309</v>
+        <v>15.45819116193756</v>
       </c>
       <c r="F39" t="n">
         <v>4653000</v>
@@ -1212,16 +1212,16 @@
         <v>44312</v>
       </c>
       <c r="B40" t="n">
-        <v>15.2606897354126</v>
+        <v>15.26068878173828</v>
       </c>
       <c r="C40" t="n">
-        <v>15.51705882313055</v>
+        <v>15.51705785343516</v>
       </c>
       <c r="D40" t="n">
-        <v>15.16573734944818</v>
+        <v>15.16573640170765</v>
       </c>
       <c r="E40" t="n">
-        <v>15.48477656941952</v>
+        <v>15.48477560174152</v>
       </c>
       <c r="F40" t="n">
         <v>3662000</v>
@@ -1232,16 +1232,16 @@
         <v>44313</v>
       </c>
       <c r="B41" t="n">
-        <v>15.12775611877441</v>
+        <v>15.1277551651001</v>
       </c>
       <c r="C41" t="n">
-        <v>15.29677114335289</v>
+        <v>15.29677017902364</v>
       </c>
       <c r="D41" t="n">
-        <v>15.10116966883617</v>
+        <v>15.1011687168379</v>
       </c>
       <c r="E41" t="n">
-        <v>15.24929404627311</v>
+        <v>15.24929308493688</v>
       </c>
       <c r="F41" t="n">
         <v>4986500</v>
@@ -1252,16 +1252,16 @@
         <v>44314</v>
       </c>
       <c r="B42" t="n">
-        <v>15.18852615356445</v>
+        <v>15.18852519989014</v>
       </c>
       <c r="C42" t="n">
-        <v>15.35564228216909</v>
+        <v>15.35564131800169</v>
       </c>
       <c r="D42" t="n">
-        <v>15.04799647598031</v>
+        <v>15.04799553112973</v>
       </c>
       <c r="E42" t="n">
-        <v>15.14864647703371</v>
+        <v>15.14864552586341</v>
       </c>
       <c r="F42" t="n">
         <v>5371500</v>
@@ -1272,16 +1272,16 @@
         <v>44315</v>
       </c>
       <c r="B43" t="n">
-        <v>15.21646499633789</v>
+        <v>15.21646595001221</v>
       </c>
       <c r="C43" t="n">
-        <v>15.32323336252505</v>
+        <v>15.32323432289095</v>
       </c>
       <c r="D43" t="n">
-        <v>14.90950503441863</v>
+        <v>14.90950596885459</v>
       </c>
       <c r="E43" t="n">
-        <v>15.26222338706449</v>
+        <v>15.26222434360666</v>
       </c>
       <c r="F43" t="n">
         <v>5343000</v>
@@ -1332,16 +1332,16 @@
         <v>44320</v>
       </c>
       <c r="B46" t="n">
-        <v>15.72933578491211</v>
+        <v>15.72933769226074</v>
       </c>
       <c r="C46" t="n">
-        <v>15.74840208285252</v>
+        <v>15.74840399251314</v>
       </c>
       <c r="D46" t="n">
-        <v>15.35945760522207</v>
+        <v>15.35945946771906</v>
       </c>
       <c r="E46" t="n">
-        <v>15.63400611347231</v>
+        <v>15.63400800926121</v>
       </c>
       <c r="F46" t="n">
         <v>9407500</v>
@@ -1412,16 +1412,16 @@
         <v>44326</v>
       </c>
       <c r="B50" t="n">
-        <v>16.81418609619141</v>
+        <v>16.81418228149414</v>
       </c>
       <c r="C50" t="n">
-        <v>17.0162841548014</v>
+        <v>17.01628029425339</v>
       </c>
       <c r="D50" t="n">
-        <v>16.55298359675715</v>
+        <v>16.55297984131987</v>
       </c>
       <c r="E50" t="n">
-        <v>16.97052576072697</v>
+        <v>16.97052191056034</v>
       </c>
       <c r="F50" t="n">
         <v>7669500</v>
@@ -1432,16 +1432,16 @@
         <v>44327</v>
       </c>
       <c r="B51" t="n">
-        <v>16.58730125427246</v>
+        <v>16.5872974395752</v>
       </c>
       <c r="C51" t="n">
-        <v>16.78368087460993</v>
+        <v>16.78367701474988</v>
       </c>
       <c r="D51" t="n">
-        <v>16.49197157097672</v>
+        <v>16.49196777820309</v>
       </c>
       <c r="E51" t="n">
-        <v>16.62543385489575</v>
+        <v>16.62543003142886</v>
       </c>
       <c r="F51" t="n">
         <v>6191000</v>
@@ -1452,16 +1452,16 @@
         <v>44328</v>
       </c>
       <c r="B52" t="n">
-        <v>16.12590789794922</v>
+        <v>16.12590599060059</v>
       </c>
       <c r="C52" t="n">
-        <v>16.57776793756821</v>
+        <v>16.57776597677424</v>
       </c>
       <c r="D52" t="n">
-        <v>16.04201690472579</v>
+        <v>16.04201500729966</v>
       </c>
       <c r="E52" t="n">
-        <v>16.49006586623571</v>
+        <v>16.49006391581501</v>
       </c>
       <c r="F52" t="n">
         <v>6728500</v>
@@ -1492,16 +1492,16 @@
         <v>44330</v>
       </c>
       <c r="B54" t="n">
-        <v>16.52628898620605</v>
+        <v>16.52629089355469</v>
       </c>
       <c r="C54" t="n">
-        <v>16.66356232925931</v>
+        <v>16.66356425245107</v>
       </c>
       <c r="D54" t="n">
-        <v>16.13734451407442</v>
+        <v>16.13734637653381</v>
       </c>
       <c r="E54" t="n">
-        <v>16.54726082268666</v>
+        <v>16.54726273245572</v>
       </c>
       <c r="F54" t="n">
         <v>5923000</v>
@@ -1532,16 +1532,16 @@
         <v>44334</v>
       </c>
       <c r="B56" t="n">
-        <v>16.06108093261719</v>
+        <v>16.06108283996582</v>
       </c>
       <c r="C56" t="n">
-        <v>16.39092096863362</v>
+        <v>16.39092291515271</v>
       </c>
       <c r="D56" t="n">
-        <v>15.88758235355229</v>
+        <v>15.88758424029694</v>
       </c>
       <c r="E56" t="n">
-        <v>16.34897547795611</v>
+        <v>16.34897741949393</v>
       </c>
       <c r="F56" t="n">
         <v>6527500</v>
@@ -1552,16 +1552,16 @@
         <v>44335</v>
       </c>
       <c r="B57" t="n">
-        <v>15.82847690582275</v>
+        <v>15.82848072052002</v>
       </c>
       <c r="C57" t="n">
-        <v>16.3680407240457</v>
+        <v>16.36804466877901</v>
       </c>
       <c r="D57" t="n">
-        <v>15.67595017276244</v>
+        <v>15.67595395070043</v>
       </c>
       <c r="E57" t="n">
-        <v>15.98481653447027</v>
+        <v>15.98482038684572</v>
       </c>
       <c r="F57" t="n">
         <v>6358000</v>
@@ -1612,16 +1612,16 @@
         <v>44340</v>
       </c>
       <c r="B60" t="n">
-        <v>17.00865364074707</v>
+        <v>17.0086555480957</v>
       </c>
       <c r="C60" t="n">
-        <v>17.06203963689752</v>
+        <v>17.06204155023285</v>
       </c>
       <c r="D60" t="n">
-        <v>16.39664113380684</v>
+        <v>16.39664297252445</v>
       </c>
       <c r="E60" t="n">
-        <v>16.5415402659626</v>
+        <v>16.54154212092919</v>
       </c>
       <c r="F60" t="n">
         <v>10386000</v>
@@ -1652,16 +1652,16 @@
         <v>44342</v>
       </c>
       <c r="B62" t="n">
-        <v>16.94192504882812</v>
+        <v>16.94192695617676</v>
       </c>
       <c r="C62" t="n">
-        <v>17.11161256574568</v>
+        <v>17.11161449219801</v>
       </c>
       <c r="D62" t="n">
-        <v>16.65975073072218</v>
+        <v>16.65975260630318</v>
       </c>
       <c r="E62" t="n">
-        <v>17.02390868058733</v>
+        <v>17.02391059716581</v>
       </c>
       <c r="F62" t="n">
         <v>5462000</v>
@@ -1672,16 +1672,16 @@
         <v>44343</v>
       </c>
       <c r="B63" t="n">
-        <v>16.94955253601074</v>
+        <v>16.94955444335938</v>
       </c>
       <c r="C63" t="n">
-        <v>17.26223183953111</v>
+        <v>17.26223378206583</v>
       </c>
       <c r="D63" t="n">
-        <v>16.70550899973091</v>
+        <v>16.7055108796171</v>
       </c>
       <c r="E63" t="n">
-        <v>16.94955253601074</v>
+        <v>16.94955444335938</v>
       </c>
       <c r="F63" t="n">
         <v>5669000</v>
@@ -1712,16 +1712,16 @@
         <v>44347</v>
       </c>
       <c r="B65" t="n">
-        <v>17.05441093444824</v>
+        <v>17.05441284179688</v>
       </c>
       <c r="C65" t="n">
-        <v>17.2546034069664</v>
+        <v>17.25460533670436</v>
       </c>
       <c r="D65" t="n">
-        <v>16.87137921937667</v>
+        <v>16.87138110625522</v>
       </c>
       <c r="E65" t="n">
-        <v>17.09254352664678</v>
+        <v>17.09254543826012</v>
       </c>
       <c r="F65" t="n">
         <v>4641000</v>
@@ -1732,16 +1732,16 @@
         <v>44348</v>
       </c>
       <c r="B66" t="n">
-        <v>16.96861839294434</v>
+        <v>16.96861457824707</v>
       </c>
       <c r="C66" t="n">
-        <v>17.41094711104222</v>
+        <v>17.4109431969055</v>
       </c>
       <c r="D66" t="n">
-        <v>16.82562477524642</v>
+        <v>16.8256209926954</v>
       </c>
       <c r="E66" t="n">
-        <v>17.17834406261295</v>
+        <v>17.17834020076747</v>
       </c>
       <c r="F66" t="n">
         <v>13722000</v>
@@ -1752,16 +1752,16 @@
         <v>44349</v>
       </c>
       <c r="B67" t="n">
-        <v>16.76652145385742</v>
+        <v>16.76651954650879</v>
       </c>
       <c r="C67" t="n">
-        <v>17.26032885279158</v>
+        <v>17.26032688926774</v>
       </c>
       <c r="D67" t="n">
-        <v>16.73982935859208</v>
+        <v>16.73982745427992</v>
       </c>
       <c r="E67" t="n">
-        <v>17.06394921675354</v>
+        <v>17.06394727556971</v>
       </c>
       <c r="F67" t="n">
         <v>9352500</v>
@@ -1772,16 +1772,16 @@
         <v>44351</v>
       </c>
       <c r="B68" t="n">
-        <v>16.77223777770996</v>
+        <v>16.77223968505859</v>
       </c>
       <c r="C68" t="n">
-        <v>16.81608880704675</v>
+        <v>16.81609071938215</v>
       </c>
       <c r="D68" t="n">
-        <v>16.40617250494436</v>
+        <v>16.40617437066384</v>
       </c>
       <c r="E68" t="n">
-        <v>16.72266649551031</v>
+        <v>16.72266839722167</v>
       </c>
       <c r="F68" t="n">
         <v>8097000</v>
@@ -1812,16 +1812,16 @@
         <v>44355</v>
       </c>
       <c r="B70" t="n">
-        <v>16.08205986022949</v>
+        <v>16.08205795288086</v>
       </c>
       <c r="C70" t="n">
-        <v>16.61018338051686</v>
+        <v>16.61018141053224</v>
       </c>
       <c r="D70" t="n">
-        <v>15.92953124909749</v>
+        <v>15.9295293598389</v>
       </c>
       <c r="E70" t="n">
-        <v>16.60065022867968</v>
+        <v>16.60064825982571</v>
       </c>
       <c r="F70" t="n">
         <v>9246000</v>
@@ -1872,16 +1872,16 @@
         <v>44358</v>
       </c>
       <c r="B73" t="n">
-        <v>16.07061386108398</v>
+        <v>16.07061576843262</v>
       </c>
       <c r="C73" t="n">
-        <v>16.30512422503518</v>
+        <v>16.30512616021678</v>
       </c>
       <c r="D73" t="n">
-        <v>15.8742360914556</v>
+        <v>15.87423797549705</v>
       </c>
       <c r="E73" t="n">
-        <v>16.30321686801416</v>
+        <v>16.3032188029694</v>
       </c>
       <c r="F73" t="n">
         <v>5133000</v>
@@ -1992,16 +1992,16 @@
         <v>44368</v>
       </c>
       <c r="B79" t="n">
-        <v>16.48434448242188</v>
+        <v>16.48434257507324</v>
       </c>
       <c r="C79" t="n">
-        <v>16.59302020374093</v>
+        <v>16.59301828381779</v>
       </c>
       <c r="D79" t="n">
-        <v>16.00007212945171</v>
+        <v>16.00007027813662</v>
       </c>
       <c r="E79" t="n">
-        <v>16.20789042268334</v>
+        <v>16.20788854732228</v>
       </c>
       <c r="F79" t="n">
         <v>6798000</v>
@@ -2032,16 +2032,16 @@
         <v>44370</v>
       </c>
       <c r="B81" t="n">
-        <v>16.39664077758789</v>
+        <v>16.39664268493652</v>
       </c>
       <c r="C81" t="n">
-        <v>16.4557433887786</v>
+        <v>16.45574530300238</v>
       </c>
       <c r="D81" t="n">
-        <v>16.20979434077605</v>
+        <v>16.20979622638967</v>
       </c>
       <c r="E81" t="n">
-        <v>16.40045367331676</v>
+        <v>16.40045558110893</v>
       </c>
       <c r="F81" t="n">
         <v>5819500</v>
@@ -2052,16 +2052,16 @@
         <v>44371</v>
       </c>
       <c r="B82" t="n">
-        <v>16.64640426635742</v>
+        <v>16.64640045166016</v>
       </c>
       <c r="C82" t="n">
-        <v>16.72648053888243</v>
+        <v>16.72647670583486</v>
       </c>
       <c r="D82" t="n">
-        <v>16.39664229944431</v>
+        <v>16.39663854198261</v>
       </c>
       <c r="E82" t="n">
-        <v>16.46909096154148</v>
+        <v>16.46908718747741</v>
       </c>
       <c r="F82" t="n">
         <v>8527500</v>
@@ -2072,16 +2072,16 @@
         <v>44372</v>
       </c>
       <c r="B83" t="n">
-        <v>16.18501091003418</v>
+        <v>16.18500900268555</v>
       </c>
       <c r="C83" t="n">
-        <v>16.74745398613881</v>
+        <v>16.74745201250817</v>
       </c>
       <c r="D83" t="n">
-        <v>16.05345599637458</v>
+        <v>16.05345410452925</v>
       </c>
       <c r="E83" t="n">
-        <v>16.64640405902371</v>
+        <v>16.64640209730146</v>
       </c>
       <c r="F83" t="n">
         <v>6078000</v>
@@ -2132,16 +2132,16 @@
         <v>44377</v>
       </c>
       <c r="B86" t="n">
-        <v>16.49959945678711</v>
+        <v>16.49959754943848</v>
       </c>
       <c r="C86" t="n">
-        <v>16.49959945678711</v>
+        <v>16.49959754943848</v>
       </c>
       <c r="D86" t="n">
-        <v>16.19073120503556</v>
+        <v>16.19072933339201</v>
       </c>
       <c r="E86" t="n">
-        <v>16.38901636774828</v>
+        <v>16.38901447318302</v>
       </c>
       <c r="F86" t="n">
         <v>6685000</v>
@@ -2172,16 +2172,16 @@
         <v>44379</v>
       </c>
       <c r="B88" t="n">
-        <v>16.39664077758789</v>
+        <v>16.39664268493652</v>
       </c>
       <c r="C88" t="n">
-        <v>16.45765074577411</v>
+        <v>16.45765266021977</v>
       </c>
       <c r="D88" t="n">
-        <v>16.21551459350043</v>
+        <v>16.21551647977946</v>
       </c>
       <c r="E88" t="n">
-        <v>16.36804133222814</v>
+        <v>16.36804323624992</v>
       </c>
       <c r="F88" t="n">
         <v>5948000</v>
@@ -2232,16 +2232,16 @@
         <v>44384</v>
       </c>
       <c r="B91" t="n">
-        <v>16.44430541992188</v>
+        <v>16.44430732727051</v>
       </c>
       <c r="C91" t="n">
-        <v>16.58348612054724</v>
+        <v>16.58348804403921</v>
       </c>
       <c r="D91" t="n">
-        <v>16.15069061682722</v>
+        <v>16.15069249011994</v>
       </c>
       <c r="E91" t="n">
-        <v>16.39664149383569</v>
+        <v>16.39664339565586</v>
       </c>
       <c r="F91" t="n">
         <v>12086500</v>
@@ -2272,16 +2272,16 @@
         <v>44389</v>
       </c>
       <c r="B93" t="n">
-        <v>16.50150299072266</v>
+        <v>16.50150489807129</v>
       </c>
       <c r="C93" t="n">
-        <v>16.60255291716791</v>
+        <v>16.60255483619654</v>
       </c>
       <c r="D93" t="n">
-        <v>16.2746202228983</v>
+        <v>16.27462210402238</v>
       </c>
       <c r="E93" t="n">
-        <v>16.43095986888196</v>
+        <v>16.43096176807677</v>
       </c>
       <c r="F93" t="n">
         <v>4327500</v>
@@ -2312,16 +2312,16 @@
         <v>44391</v>
       </c>
       <c r="B95" t="n">
-        <v>16.7226676940918</v>
+        <v>16.72266578674316</v>
       </c>
       <c r="C95" t="n">
-        <v>17.08873299309478</v>
+        <v>17.08873104399359</v>
       </c>
       <c r="D95" t="n">
-        <v>16.67309640833917</v>
+        <v>16.67309450664453</v>
       </c>
       <c r="E95" t="n">
-        <v>16.9304859864696</v>
+        <v>16.9304840554177</v>
       </c>
       <c r="F95" t="n">
         <v>5548000</v>
@@ -2332,16 +2332,16 @@
         <v>44392</v>
       </c>
       <c r="B96" t="n">
-        <v>16.45002555847168</v>
+        <v>16.45002746582031</v>
       </c>
       <c r="C96" t="n">
-        <v>16.86375476157448</v>
+        <v>16.86375671689422</v>
       </c>
       <c r="D96" t="n">
-        <v>16.44049240966831</v>
+        <v>16.44049431591159</v>
       </c>
       <c r="E96" t="n">
-        <v>16.72266670485169</v>
+        <v>16.72266864381253</v>
       </c>
       <c r="F96" t="n">
         <v>3746000</v>
@@ -2432,16 +2432,16 @@
         <v>44399</v>
       </c>
       <c r="B101" t="n">
-        <v>16.64449882507324</v>
+        <v>16.64449691772461</v>
       </c>
       <c r="C101" t="n">
-        <v>16.68072406942274</v>
+        <v>16.68072215792294</v>
       </c>
       <c r="D101" t="n">
-        <v>16.44430812071748</v>
+        <v>16.44430623630937</v>
       </c>
       <c r="E101" t="n">
-        <v>16.58730174072338</v>
+        <v>16.58729983992916</v>
       </c>
       <c r="F101" t="n">
         <v>2829500</v>
@@ -2452,16 +2452,16 @@
         <v>44400</v>
       </c>
       <c r="B102" t="n">
-        <v>16.68263053894043</v>
+        <v>16.68263244628906</v>
       </c>
       <c r="C102" t="n">
-        <v>16.73029447031815</v>
+        <v>16.73029638311626</v>
       </c>
       <c r="D102" t="n">
-        <v>16.56060876542906</v>
+        <v>16.56061065882677</v>
       </c>
       <c r="E102" t="n">
-        <v>16.64449793922831</v>
+        <v>16.64449984221719</v>
       </c>
       <c r="F102" t="n">
         <v>4154500</v>
@@ -2492,16 +2492,16 @@
         <v>44404</v>
       </c>
       <c r="B104" t="n">
-        <v>16.96861839294434</v>
+        <v>16.96861457824707</v>
       </c>
       <c r="C104" t="n">
-        <v>17.300365840649</v>
+        <v>17.30036195137194</v>
       </c>
       <c r="D104" t="n">
-        <v>16.87329052665406</v>
+        <v>16.87328673338735</v>
       </c>
       <c r="E104" t="n">
-        <v>17.14402435794695</v>
+        <v>17.14402050381685</v>
       </c>
       <c r="F104" t="n">
         <v>6666500</v>
@@ -2512,16 +2512,16 @@
         <v>44405</v>
       </c>
       <c r="B105" t="n">
-        <v>16.79321098327637</v>
+        <v>16.793212890625</v>
       </c>
       <c r="C105" t="n">
-        <v>17.38044062591602</v>
+        <v>17.38044259996134</v>
       </c>
       <c r="D105" t="n">
-        <v>16.42333460278985</v>
+        <v>16.42333646812846</v>
       </c>
       <c r="E105" t="n">
-        <v>17.34993563859687</v>
+        <v>17.34993760917749</v>
       </c>
       <c r="F105" t="n">
         <v>14614500</v>
@@ -2552,16 +2552,16 @@
         <v>44407</v>
       </c>
       <c r="B107" t="n">
-        <v>16.52628898620605</v>
+        <v>16.52629089355469</v>
       </c>
       <c r="C107" t="n">
-        <v>16.73219990991705</v>
+        <v>16.73220184103048</v>
       </c>
       <c r="D107" t="n">
-        <v>16.30893755658766</v>
+        <v>16.30893943885111</v>
       </c>
       <c r="E107" t="n">
-        <v>16.62543155217983</v>
+        <v>16.6254334709708</v>
       </c>
       <c r="F107" t="n">
         <v>16469000</v>
@@ -2612,16 +2612,16 @@
         <v>44412</v>
       </c>
       <c r="B110" t="n">
-        <v>16.60255432128906</v>
+        <v>16.6025505065918</v>
       </c>
       <c r="C110" t="n">
-        <v>16.83134446559894</v>
+        <v>16.83134059833355</v>
       </c>
       <c r="D110" t="n">
-        <v>16.3489776234245</v>
+        <v>16.34897386699046</v>
       </c>
       <c r="E110" t="n">
-        <v>16.48243990463543</v>
+        <v>16.48243611753633</v>
       </c>
       <c r="F110" t="n">
         <v>6533500</v>
@@ -2632,16 +2632,16 @@
         <v>44413</v>
       </c>
       <c r="B111" t="n">
-        <v>16.58730125427246</v>
+        <v>16.5872974395752</v>
       </c>
       <c r="C111" t="n">
-        <v>16.93811317965181</v>
+        <v>16.93810928427588</v>
       </c>
       <c r="D111" t="n">
-        <v>16.47481262800123</v>
+        <v>16.47480883917376</v>
       </c>
       <c r="E111" t="n">
-        <v>16.59302150801845</v>
+        <v>16.59301769200566</v>
       </c>
       <c r="F111" t="n">
         <v>13427000</v>
@@ -2652,16 +2652,16 @@
         <v>44414</v>
       </c>
       <c r="B112" t="n">
-        <v>16.73983001708984</v>
+        <v>16.73982810974121</v>
       </c>
       <c r="C112" t="n">
-        <v>16.78368287669021</v>
+        <v>16.78368096434495</v>
       </c>
       <c r="D112" t="n">
-        <v>16.37567200170541</v>
+        <v>16.37567013584921</v>
       </c>
       <c r="E112" t="n">
-        <v>16.63115427426481</v>
+        <v>16.63115237929877</v>
       </c>
       <c r="F112" t="n">
         <v>15424500</v>
@@ -2672,16 +2672,16 @@
         <v>44417</v>
       </c>
       <c r="B113" t="n">
-        <v>17.31942749023438</v>
+        <v>17.31942939758301</v>
       </c>
       <c r="C113" t="n">
-        <v>17.35756008512363</v>
+        <v>17.35756199667172</v>
       </c>
       <c r="D113" t="n">
-        <v>16.61780374497947</v>
+        <v>16.6178055750599</v>
       </c>
       <c r="E113" t="n">
-        <v>16.61780374497947</v>
+        <v>16.6178055750599</v>
       </c>
       <c r="F113" t="n">
         <v>10558500</v>
@@ -2692,16 +2692,16 @@
         <v>44418</v>
       </c>
       <c r="B114" t="n">
-        <v>17.55012893676758</v>
+        <v>17.55012512207031</v>
       </c>
       <c r="C114" t="n">
-        <v>17.66452492908273</v>
+        <v>17.66452108952034</v>
       </c>
       <c r="D114" t="n">
-        <v>17.10589465161376</v>
+        <v>17.10589093347529</v>
       </c>
       <c r="E114" t="n">
-        <v>17.22219618314763</v>
+        <v>17.22219243972985</v>
       </c>
       <c r="F114" t="n">
         <v>10281500</v>
@@ -2712,16 +2712,16 @@
         <v>44419</v>
       </c>
       <c r="B115" t="n">
-        <v>17.20884704589844</v>
+        <v>17.2088451385498</v>
       </c>
       <c r="C115" t="n">
-        <v>17.57872523333663</v>
+        <v>17.57872328499242</v>
       </c>
       <c r="D115" t="n">
-        <v>17.19740835785192</v>
+        <v>17.1974064517711</v>
       </c>
       <c r="E115" t="n">
-        <v>17.57872523333663</v>
+        <v>17.57872328499242</v>
       </c>
       <c r="F115" t="n">
         <v>6265000</v>
@@ -2772,16 +2772,16 @@
         <v>44424</v>
       </c>
       <c r="B118" t="n">
-        <v>16.44430541992188</v>
+        <v>16.44430732727051</v>
       </c>
       <c r="C118" t="n">
-        <v>17.04487925261408</v>
+        <v>17.04488122962231</v>
       </c>
       <c r="D118" t="n">
-        <v>16.27271237679204</v>
+        <v>16.27271426423787</v>
       </c>
       <c r="E118" t="n">
-        <v>16.86375487887679</v>
+        <v>16.86375683487669</v>
       </c>
       <c r="F118" t="n">
         <v>7814500</v>
@@ -2852,16 +2852,16 @@
         <v>44428</v>
       </c>
       <c r="B122" t="n">
-        <v>16.94955253601074</v>
+        <v>16.94955444335938</v>
       </c>
       <c r="C122" t="n">
-        <v>17.41666595234703</v>
+        <v>17.41666791226037</v>
       </c>
       <c r="D122" t="n">
-        <v>16.37757629334467</v>
+        <v>16.3775781363283</v>
       </c>
       <c r="E122" t="n">
-        <v>16.53963619846235</v>
+        <v>16.53963805968273</v>
       </c>
       <c r="F122" t="n">
         <v>9513400</v>
@@ -2872,16 +2872,16 @@
         <v>44431</v>
       </c>
       <c r="B123" t="n">
-        <v>16.69216537475586</v>
+        <v>16.69216346740723</v>
       </c>
       <c r="C123" t="n">
-        <v>17.16881200972343</v>
+        <v>17.16881004791025</v>
       </c>
       <c r="D123" t="n">
-        <v>16.52057229524551</v>
+        <v>16.52057040750415</v>
       </c>
       <c r="E123" t="n">
-        <v>16.97815262843136</v>
+        <v>16.97815068840407</v>
       </c>
       <c r="F123" t="n">
         <v>5050600</v>
@@ -2952,16 +2952,16 @@
         <v>44435</v>
       </c>
       <c r="B127" t="n">
-        <v>16.58730125427246</v>
+        <v>16.5872974395752</v>
       </c>
       <c r="C127" t="n">
-        <v>16.72076353819149</v>
+        <v>16.72075969280097</v>
       </c>
       <c r="D127" t="n">
-        <v>16.39664370594345</v>
+        <v>16.39663993509303</v>
       </c>
       <c r="E127" t="n">
-        <v>16.55870362206747</v>
+        <v>16.558699813947</v>
       </c>
       <c r="F127" t="n">
         <v>5662600</v>
@@ -2992,16 +2992,16 @@
         <v>44439</v>
       </c>
       <c r="B129" t="n">
-        <v>16.02485847473145</v>
+        <v>16.02485656738281</v>
       </c>
       <c r="C129" t="n">
-        <v>16.63496737026124</v>
+        <v>16.63496539029478</v>
       </c>
       <c r="D129" t="n">
-        <v>16.02485847473145</v>
+        <v>16.02485656738281</v>
       </c>
       <c r="E129" t="n">
-        <v>16.37757776519067</v>
+        <v>16.37757581585984</v>
       </c>
       <c r="F129" t="n">
         <v>8477100</v>
@@ -3012,16 +3012,16 @@
         <v>44440</v>
       </c>
       <c r="B130" t="n">
-        <v>16.23458290100098</v>
+        <v>16.23458480834961</v>
       </c>
       <c r="C130" t="n">
-        <v>16.77795970229644</v>
+        <v>16.77796167348466</v>
       </c>
       <c r="D130" t="n">
-        <v>15.89139678723021</v>
+        <v>15.89139865425901</v>
       </c>
       <c r="E130" t="n">
-        <v>16.30131313017587</v>
+        <v>16.30131504536443</v>
       </c>
       <c r="F130" t="n">
         <v>7651500</v>
@@ -3032,16 +3032,16 @@
         <v>44441</v>
       </c>
       <c r="B131" t="n">
-        <v>16.72076225280762</v>
+        <v>16.72076416015625</v>
       </c>
       <c r="C131" t="n">
-        <v>17.03534891071645</v>
+        <v>17.03535085395019</v>
       </c>
       <c r="D131" t="n">
-        <v>16.10112026815059</v>
+        <v>16.10112210481625</v>
       </c>
       <c r="E131" t="n">
-        <v>16.16785049584908</v>
+        <v>16.1678523401267</v>
       </c>
       <c r="F131" t="n">
         <v>17566400</v>
@@ -3072,16 +3072,16 @@
         <v>44445</v>
       </c>
       <c r="B133" t="n">
-        <v>17.49292945861816</v>
+        <v>17.4929313659668</v>
       </c>
       <c r="C133" t="n">
-        <v>17.66452251450438</v>
+        <v>17.66452444056273</v>
       </c>
       <c r="D133" t="n">
-        <v>17.04488051974584</v>
+        <v>17.04488237824128</v>
       </c>
       <c r="E133" t="n">
-        <v>17.30227010357517</v>
+        <v>17.30227199013519</v>
       </c>
       <c r="F133" t="n">
         <v>6471000</v>
@@ -3212,16 +3212,16 @@
         <v>44455</v>
       </c>
       <c r="B140" t="n">
-        <v>18.26509857177734</v>
+        <v>18.26509666442871</v>
       </c>
       <c r="C140" t="n">
-        <v>18.33182880852791</v>
+        <v>18.33182689421092</v>
       </c>
       <c r="D140" t="n">
-        <v>17.72172170879404</v>
+        <v>17.72171985818801</v>
       </c>
       <c r="E140" t="n">
-        <v>17.72172170879404</v>
+        <v>17.72171985818801</v>
       </c>
       <c r="F140" t="n">
         <v>17281800</v>
@@ -3232,16 +3232,16 @@
         <v>44456</v>
       </c>
       <c r="B141" t="n">
-        <v>18.11257171630859</v>
+        <v>18.11256980895996</v>
       </c>
       <c r="C141" t="n">
-        <v>18.44622471684048</v>
+        <v>18.44622277435644</v>
       </c>
       <c r="D141" t="n">
-        <v>18.11257171630859</v>
+        <v>18.11256980895996</v>
       </c>
       <c r="E141" t="n">
-        <v>18.28416479191142</v>
+        <v>18.28416286649314</v>
       </c>
       <c r="F141" t="n">
         <v>23104900</v>
@@ -3252,16 +3252,16 @@
         <v>44459</v>
       </c>
       <c r="B142" t="n">
-        <v>17.94097709655762</v>
+        <v>17.94097900390625</v>
       </c>
       <c r="C142" t="n">
-        <v>18.12210330724501</v>
+        <v>18.12210523384961</v>
       </c>
       <c r="D142" t="n">
-        <v>17.63592357430248</v>
+        <v>17.63592544922014</v>
       </c>
       <c r="E142" t="n">
-        <v>18.02677362697468</v>
+        <v>18.02677554344455</v>
       </c>
       <c r="F142" t="n">
         <v>15522000</v>
@@ -3312,16 +3312,16 @@
         <v>44462</v>
       </c>
       <c r="B145" t="n">
-        <v>18.29369735717773</v>
+        <v>18.2936954498291</v>
       </c>
       <c r="C145" t="n">
-        <v>18.53202066160796</v>
+        <v>18.53201872941112</v>
       </c>
       <c r="D145" t="n">
-        <v>18.07443853522241</v>
+        <v>18.07443665073428</v>
       </c>
       <c r="E145" t="n">
-        <v>18.34136129075877</v>
+        <v>18.34135937844058</v>
       </c>
       <c r="F145" t="n">
         <v>20822300</v>
@@ -3332,16 +3332,16 @@
         <v>44463</v>
       </c>
       <c r="B146" t="n">
-        <v>18.09350395202637</v>
+        <v>18.09350204467773</v>
       </c>
       <c r="C146" t="n">
-        <v>18.26509701375519</v>
+        <v>18.26509508831786</v>
       </c>
       <c r="D146" t="n">
-        <v>17.87424695904506</v>
+        <v>17.87424507480967</v>
       </c>
       <c r="E146" t="n">
-        <v>18.13163655163829</v>
+        <v>18.13163464026987</v>
       </c>
       <c r="F146" t="n">
         <v>18657800</v>
@@ -3372,16 +3372,16 @@
         <v>44467</v>
       </c>
       <c r="B148" t="n">
-        <v>18.28416061401367</v>
+        <v>18.2841625213623</v>
       </c>
       <c r="C148" t="n">
-        <v>18.29369376250914</v>
+        <v>18.29369567085224</v>
       </c>
       <c r="D148" t="n">
-        <v>18.01723791092701</v>
+        <v>18.01723979043107</v>
       </c>
       <c r="E148" t="n">
-        <v>18.23649487153633</v>
+        <v>18.23649677391261</v>
       </c>
       <c r="F148" t="n">
         <v>11310100</v>
@@ -3412,16 +3412,16 @@
         <v>44469</v>
       </c>
       <c r="B150" t="n">
-        <v>18.15070152282715</v>
+        <v>18.15070343017578</v>
       </c>
       <c r="C150" t="n">
-        <v>18.62734807351153</v>
+        <v>18.6273500309481</v>
       </c>
       <c r="D150" t="n">
-        <v>18.04583869983265</v>
+        <v>18.04584059616188</v>
       </c>
       <c r="E150" t="n">
-        <v>18.30322827358517</v>
+        <v>18.30323019696192</v>
       </c>
       <c r="F150" t="n">
         <v>10293000</v>
@@ -3472,16 +3472,16 @@
         <v>44474</v>
       </c>
       <c r="B153" t="n">
-        <v>18.32229423522949</v>
+        <v>18.32229232788086</v>
       </c>
       <c r="C153" t="n">
-        <v>18.49388729827244</v>
+        <v>18.49388537306099</v>
       </c>
       <c r="D153" t="n">
-        <v>18.04584015897554</v>
+        <v>18.04583828040574</v>
       </c>
       <c r="E153" t="n">
-        <v>18.34136053518147</v>
+        <v>18.34135862584804</v>
       </c>
       <c r="F153" t="n">
         <v>8000200</v>
@@ -3492,16 +3492,16 @@
         <v>44475</v>
       </c>
       <c r="B154" t="n">
-        <v>18.27167510986328</v>
+        <v>18.27167892456055</v>
       </c>
       <c r="C154" t="n">
-        <v>18.63481427841922</v>
+        <v>18.63481816893143</v>
       </c>
       <c r="D154" t="n">
-        <v>18.0614350130003</v>
+        <v>18.06143878380436</v>
       </c>
       <c r="E154" t="n">
-        <v>18.11877239272545</v>
+        <v>18.11877617550022</v>
       </c>
       <c r="F154" t="n">
         <v>10611600</v>
@@ -3552,16 +3552,16 @@
         <v>44480</v>
       </c>
       <c r="B157" t="n">
-        <v>16.62799072265625</v>
+        <v>16.62798881530762</v>
       </c>
       <c r="C157" t="n">
-        <v>17.52628500439614</v>
+        <v>17.52628299400677</v>
       </c>
       <c r="D157" t="n">
-        <v>16.47508980100556</v>
+        <v>16.47508791119575</v>
       </c>
       <c r="E157" t="n">
-        <v>17.42116493724025</v>
+        <v>17.4211629389089</v>
       </c>
       <c r="F157" t="n">
         <v>31512800</v>
@@ -3632,16 +3632,16 @@
         <v>44487</v>
       </c>
       <c r="B161" t="n">
-        <v>16.20751190185547</v>
+        <v>16.20750999450684</v>
       </c>
       <c r="C161" t="n">
-        <v>16.67577301414236</v>
+        <v>16.67577105168735</v>
       </c>
       <c r="D161" t="n">
-        <v>16.10239365985386</v>
+        <v>16.10239176487586</v>
       </c>
       <c r="E161" t="n">
-        <v>16.58976601986295</v>
+        <v>16.5897640675295</v>
       </c>
       <c r="F161" t="n">
         <v>13070300</v>
@@ -3692,16 +3692,16 @@
         <v>44490</v>
       </c>
       <c r="B164" t="n">
-        <v>15.70102977752686</v>
+        <v>15.70102787017822</v>
       </c>
       <c r="C164" t="n">
-        <v>16.21706996923507</v>
+        <v>16.21706799919828</v>
       </c>
       <c r="D164" t="n">
-        <v>15.31877744612764</v>
+        <v>15.31877558521472</v>
       </c>
       <c r="E164" t="n">
-        <v>15.81570456558517</v>
+        <v>15.81570264430594</v>
       </c>
       <c r="F164" t="n">
         <v>11995800</v>
@@ -3732,16 +3732,16 @@
         <v>44494</v>
       </c>
       <c r="B166" t="n">
-        <v>15.41433715820312</v>
+        <v>15.41433811187744</v>
       </c>
       <c r="C166" t="n">
-        <v>15.66280159699508</v>
+        <v>15.66280256604172</v>
       </c>
       <c r="D166" t="n">
-        <v>15.1372049374846</v>
+        <v>15.13720587401294</v>
       </c>
       <c r="E166" t="n">
-        <v>15.39522591115963</v>
+        <v>15.39522686365155</v>
       </c>
       <c r="F166" t="n">
         <v>20484500</v>
@@ -3752,16 +3752,16 @@
         <v>44495</v>
       </c>
       <c r="B167" t="n">
-        <v>15.24232387542725</v>
+        <v>15.24232482910156</v>
       </c>
       <c r="C167" t="n">
-        <v>15.44300654837805</v>
+        <v>15.44300751460859</v>
       </c>
       <c r="D167" t="n">
-        <v>15.0129725095867</v>
+        <v>15.01297344891107</v>
       </c>
       <c r="E167" t="n">
-        <v>15.38566916259858</v>
+        <v>15.38567012524165</v>
       </c>
       <c r="F167" t="n">
         <v>7090300</v>
@@ -3812,16 +3812,16 @@
         <v>44498</v>
       </c>
       <c r="B170" t="n">
-        <v>14.61160659790039</v>
+        <v>14.61160755157471</v>
       </c>
       <c r="C170" t="n">
-        <v>15.21365459344056</v>
+        <v>15.21365558640951</v>
       </c>
       <c r="D170" t="n">
-        <v>14.50648745380085</v>
+        <v>14.50648840061422</v>
       </c>
       <c r="E170" t="n">
-        <v>15.0034153938802</v>
+        <v>15.0034163731272</v>
       </c>
       <c r="F170" t="n">
         <v>13706000</v>
@@ -3832,16 +3832,16 @@
         <v>44501</v>
       </c>
       <c r="B171" t="n">
-        <v>14.31536102294922</v>
+        <v>14.31536197662354</v>
       </c>
       <c r="C171" t="n">
-        <v>14.77406466781794</v>
+        <v>14.77406565205061</v>
       </c>
       <c r="D171" t="n">
-        <v>14.20068533957237</v>
+        <v>14.20068628560711</v>
       </c>
       <c r="E171" t="n">
-        <v>14.76450813302954</v>
+        <v>14.76450911662556</v>
       </c>
       <c r="F171" t="n">
         <v>10277500</v>
@@ -3852,16 +3852,16 @@
         <v>44503</v>
       </c>
       <c r="B172" t="n">
-        <v>14.74539661407471</v>
+        <v>14.74539566040039</v>
       </c>
       <c r="C172" t="n">
-        <v>14.86962883762583</v>
+        <v>14.86962787591666</v>
       </c>
       <c r="D172" t="n">
-        <v>14.07645373166693</v>
+        <v>14.07645282125721</v>
       </c>
       <c r="E172" t="n">
-        <v>14.14334856672452</v>
+        <v>14.14334765198831</v>
       </c>
       <c r="F172" t="n">
         <v>21906500</v>
@@ -3872,16 +3872,16 @@
         <v>44504</v>
       </c>
       <c r="B173" t="n">
-        <v>14.52560138702393</v>
+        <v>14.52560043334961</v>
       </c>
       <c r="C173" t="n">
-        <v>14.73584061228703</v>
+        <v>14.73583964480952</v>
       </c>
       <c r="D173" t="n">
-        <v>14.30580653757357</v>
+        <v>14.30580559832982</v>
       </c>
       <c r="E173" t="n">
-        <v>14.69761538145387</v>
+        <v>14.69761441648602</v>
       </c>
       <c r="F173" t="n">
         <v>4262500</v>
@@ -3892,16 +3892,16 @@
         <v>44505</v>
       </c>
       <c r="B174" t="n">
-        <v>14.5638256072998</v>
+        <v>14.56382656097412</v>
       </c>
       <c r="C174" t="n">
-        <v>14.71672652002295</v>
+        <v>14.71672748370959</v>
       </c>
       <c r="D174" t="n">
-        <v>14.1720167906064</v>
+        <v>14.17201771862414</v>
       </c>
       <c r="E174" t="n">
-        <v>14.54471344889008</v>
+        <v>14.54471440131288</v>
       </c>
       <c r="F174" t="n">
         <v>8161700</v>
@@ -3952,16 +3952,16 @@
         <v>44510</v>
       </c>
       <c r="B177" t="n">
-        <v>15.26143741607666</v>
+        <v>15.26143836975098</v>
       </c>
       <c r="C177" t="n">
-        <v>15.38566963758256</v>
+        <v>15.38567059902005</v>
       </c>
       <c r="D177" t="n">
-        <v>14.71672676618749</v>
+        <v>14.7167276858233</v>
       </c>
       <c r="E177" t="n">
-        <v>14.84095898769339</v>
+        <v>14.84095991509237</v>
       </c>
       <c r="F177" t="n">
         <v>10223900</v>
@@ -3972,16 +3972,16 @@
         <v>44511</v>
       </c>
       <c r="B178" t="n">
-        <v>15.19454193115234</v>
+        <v>15.19454288482666</v>
       </c>
       <c r="C178" t="n">
-        <v>15.51945681788442</v>
+        <v>15.51945779195179</v>
       </c>
       <c r="D178" t="n">
-        <v>15.07986624960478</v>
+        <v>15.07986719608156</v>
       </c>
       <c r="E178" t="n">
-        <v>15.43344982888343</v>
+        <v>15.43345079755262</v>
       </c>
       <c r="F178" t="n">
         <v>5555700</v>
@@ -4012,16 +4012,16 @@
         <v>44516</v>
       </c>
       <c r="B180" t="n">
-        <v>14.18157291412354</v>
+        <v>14.18157386779785</v>
       </c>
       <c r="C180" t="n">
-        <v>14.86007137817213</v>
+        <v>14.86007237747372</v>
       </c>
       <c r="D180" t="n">
-        <v>14.00000240201066</v>
+        <v>14.00000334347483</v>
       </c>
       <c r="E180" t="n">
-        <v>14.81228961649183</v>
+        <v>14.81229061258022</v>
       </c>
       <c r="F180" t="n">
         <v>11424100</v>
@@ -4032,16 +4032,16 @@
         <v>44517</v>
       </c>
       <c r="B181" t="n">
-        <v>13.62730693817139</v>
+        <v>13.62730598449707</v>
       </c>
       <c r="C181" t="n">
-        <v>14.42048109928345</v>
+        <v>14.42048009010075</v>
       </c>
       <c r="D181" t="n">
-        <v>13.49351818506572</v>
+        <v>13.49351724075429</v>
       </c>
       <c r="E181" t="n">
-        <v>14.42048109928345</v>
+        <v>14.42048009010075</v>
       </c>
       <c r="F181" t="n">
         <v>10535200</v>
@@ -4072,16 +4072,16 @@
         <v>44519</v>
       </c>
       <c r="B183" t="n">
-        <v>13.45529365539551</v>
+        <v>13.45529460906982</v>
       </c>
       <c r="C183" t="n">
-        <v>13.74198333471972</v>
+        <v>13.74198430871382</v>
       </c>
       <c r="D183" t="n">
-        <v>13.28327966552871</v>
+        <v>13.28328060701114</v>
       </c>
       <c r="E183" t="n">
-        <v>13.35017450123322</v>
+        <v>13.35017544745698</v>
       </c>
       <c r="F183" t="n">
         <v>11060800</v>
@@ -4132,16 +4132,16 @@
         <v>44524</v>
       </c>
       <c r="B186" t="n">
-        <v>13.11126613616943</v>
+        <v>13.11126518249512</v>
       </c>
       <c r="C186" t="n">
-        <v>13.38839927066881</v>
+        <v>13.38839829683666</v>
       </c>
       <c r="D186" t="n">
-        <v>12.97747738072233</v>
+        <v>12.97747643677941</v>
       </c>
       <c r="E186" t="n">
-        <v>13.09215306623642</v>
+        <v>13.09215211395233</v>
       </c>
       <c r="F186" t="n">
         <v>5705900</v>
@@ -4172,16 +4172,16 @@
         <v>44526</v>
       </c>
       <c r="B188" t="n">
-        <v>12.76723766326904</v>
+        <v>12.76723861694336</v>
       </c>
       <c r="C188" t="n">
-        <v>13.02525862899095</v>
+        <v>13.02525960193866</v>
       </c>
       <c r="D188" t="n">
-        <v>12.64300544770234</v>
+        <v>12.64300639209688</v>
       </c>
       <c r="E188" t="n">
-        <v>12.93925164041698</v>
+        <v>12.93925260694023</v>
       </c>
       <c r="F188" t="n">
         <v>6311300</v>
@@ -4212,16 +4212,16 @@
         <v>44530</v>
       </c>
       <c r="B190" t="n">
-        <v>12.18430328369141</v>
+        <v>12.18430233001709</v>
       </c>
       <c r="C190" t="n">
-        <v>12.44232426127008</v>
+        <v>12.44232328740027</v>
       </c>
       <c r="D190" t="n">
-        <v>11.84027622494785</v>
+        <v>11.84027529820078</v>
       </c>
       <c r="E190" t="n">
-        <v>12.38498596246548</v>
+        <v>12.38498499308359</v>
       </c>
       <c r="F190" t="n">
         <v>16793700</v>
@@ -4232,16 +4232,16 @@
         <v>44531</v>
       </c>
       <c r="B191" t="n">
-        <v>11.91672706604004</v>
+        <v>11.91672611236572</v>
       </c>
       <c r="C191" t="n">
-        <v>12.37542982579687</v>
+        <v>12.37542883541339</v>
       </c>
       <c r="D191" t="n">
-        <v>11.81160700007474</v>
+        <v>11.81160605481299</v>
       </c>
       <c r="E191" t="n">
-        <v>12.2989793658374</v>
+        <v>12.29897838157211</v>
       </c>
       <c r="F191" t="n">
         <v>5991300</v>
@@ -4252,16 +4252,16 @@
         <v>44532</v>
       </c>
       <c r="B192" t="n">
-        <v>11.89761257171631</v>
+        <v>11.89761352539062</v>
       </c>
       <c r="C192" t="n">
-        <v>12.14607699253434</v>
+        <v>12.14607796612476</v>
       </c>
       <c r="D192" t="n">
-        <v>11.71604297887929</v>
+        <v>11.71604391799958</v>
       </c>
       <c r="E192" t="n">
-        <v>12.14607699253434</v>
+        <v>12.14607796612476</v>
       </c>
       <c r="F192" t="n">
         <v>7306700</v>
@@ -4272,16 +4272,16 @@
         <v>44533</v>
       </c>
       <c r="B193" t="n">
-        <v>12.70990180969238</v>
+        <v>12.70990085601807</v>
       </c>
       <c r="C193" t="n">
-        <v>12.74812704129032</v>
+        <v>12.74812608474781</v>
       </c>
       <c r="D193" t="n">
-        <v>11.95495280211211</v>
+        <v>11.95495190508461</v>
       </c>
       <c r="E193" t="n">
-        <v>11.99317803371005</v>
+        <v>11.99317713381436</v>
       </c>
       <c r="F193" t="n">
         <v>16852000</v>
@@ -4312,16 +4312,16 @@
         <v>44537</v>
       </c>
       <c r="B195" t="n">
-        <v>13.42662620544434</v>
+        <v>13.4266242980957</v>
       </c>
       <c r="C195" t="n">
-        <v>13.76109676952499</v>
+        <v>13.76109481466241</v>
       </c>
       <c r="D195" t="n">
-        <v>13.40751313308241</v>
+        <v>13.40751122844893</v>
       </c>
       <c r="E195" t="n">
-        <v>13.56997060271298</v>
+        <v>13.56996867500125</v>
       </c>
       <c r="F195" t="n">
         <v>14090400</v>
@@ -4352,16 +4352,16 @@
         <v>44539</v>
       </c>
       <c r="B197" t="n">
-        <v>13.58908271789551</v>
+        <v>13.58908176422119</v>
       </c>
       <c r="C197" t="n">
-        <v>13.74198364057517</v>
+        <v>13.74198267617036</v>
       </c>
       <c r="D197" t="n">
-        <v>13.43618179521584</v>
+        <v>13.43618085227203</v>
       </c>
       <c r="E197" t="n">
-        <v>13.74198364057517</v>
+        <v>13.74198267617036</v>
       </c>
       <c r="F197" t="n">
         <v>9843600</v>
@@ -4452,16 +4452,16 @@
         <v>44546</v>
       </c>
       <c r="B202" t="n">
-        <v>13.89488315582275</v>
+        <v>13.89488410949707</v>
       </c>
       <c r="C202" t="n">
-        <v>14.28669195834289</v>
+        <v>14.28669293890897</v>
       </c>
       <c r="D202" t="n">
-        <v>13.82798923676653</v>
+        <v>13.82799018584958</v>
       </c>
       <c r="E202" t="n">
-        <v>14.21024150474683</v>
+        <v>14.21024248006574</v>
       </c>
       <c r="F202" t="n">
         <v>5287600</v>
@@ -4472,16 +4472,16 @@
         <v>44547</v>
       </c>
       <c r="B203" t="n">
-        <v>13.81843280792236</v>
+        <v>13.81843376159668</v>
       </c>
       <c r="C203" t="n">
-        <v>14.00955894337442</v>
+        <v>14.00955991023924</v>
       </c>
       <c r="D203" t="n">
-        <v>13.64641883033486</v>
+        <v>13.6464197721377</v>
       </c>
       <c r="E203" t="n">
-        <v>13.84710150039985</v>
+        <v>13.84710245605272</v>
       </c>
       <c r="F203" t="n">
         <v>8250000</v>
@@ -4492,16 +4492,16 @@
         <v>44550</v>
       </c>
       <c r="B204" t="n">
-        <v>13.47440719604492</v>
+        <v>13.47440624237061</v>
       </c>
       <c r="C204" t="n">
-        <v>13.8662160431998</v>
+        <v>13.86621506179454</v>
       </c>
       <c r="D204" t="n">
-        <v>13.29283666454885</v>
+        <v>13.29283572372549</v>
       </c>
       <c r="E204" t="n">
-        <v>13.81843427641866</v>
+        <v>13.81843329839523</v>
       </c>
       <c r="F204" t="n">
         <v>6680500</v>
@@ -4512,16 +4512,16 @@
         <v>44551</v>
       </c>
       <c r="B205" t="n">
-        <v>13.617751121521</v>
+        <v>13.61775207519531</v>
       </c>
       <c r="C205" t="n">
-        <v>13.6655328866758</v>
+        <v>13.66553384369636</v>
       </c>
       <c r="D205" t="n">
-        <v>13.36928667180511</v>
+        <v>13.36928760807904</v>
       </c>
       <c r="E205" t="n">
-        <v>13.48396236135982</v>
+        <v>13.48396330566468</v>
       </c>
       <c r="F205" t="n">
         <v>4083800</v>
@@ -4532,16 +4532,16 @@
         <v>44552</v>
       </c>
       <c r="B206" t="n">
-        <v>13.53174304962158</v>
+        <v>13.5317440032959</v>
       </c>
       <c r="C206" t="n">
-        <v>13.66553179913548</v>
+        <v>13.66553276223881</v>
       </c>
       <c r="D206" t="n">
-        <v>13.29283515422187</v>
+        <v>13.29283609105872</v>
       </c>
       <c r="E206" t="n">
-        <v>13.58908134551648</v>
+        <v>13.58908230323182</v>
       </c>
       <c r="F206" t="n">
         <v>6990400</v>
@@ -4552,16 +4552,16 @@
         <v>44553</v>
       </c>
       <c r="B207" t="n">
-        <v>13.4648494720459</v>
+        <v>13.46484851837158</v>
       </c>
       <c r="C207" t="n">
-        <v>13.65597561094082</v>
+        <v>13.65597464372962</v>
       </c>
       <c r="D207" t="n">
-        <v>13.32150418435372</v>
+        <v>13.32150324083211</v>
       </c>
       <c r="E207" t="n">
-        <v>13.41706770948184</v>
+        <v>13.41706675919176</v>
       </c>
       <c r="F207" t="n">
         <v>4198000</v>
@@ -4692,16 +4692,16 @@
         <v>44566</v>
       </c>
       <c r="B214" t="n">
-        <v>11.45802307128906</v>
+        <v>11.45802402496338</v>
       </c>
       <c r="C214" t="n">
-        <v>12.13652156778615</v>
+        <v>12.13652257793327</v>
       </c>
       <c r="D214" t="n">
-        <v>11.41024130732365</v>
+        <v>11.41024225702099</v>
       </c>
       <c r="E214" t="n">
-        <v>12.1174094090168</v>
+        <v>12.11741041757316</v>
       </c>
       <c r="F214" t="n">
         <v>11220000</v>
@@ -4712,16 +4712,16 @@
         <v>44567</v>
       </c>
       <c r="B215" t="n">
-        <v>11.07577133178711</v>
+        <v>11.07577037811279</v>
       </c>
       <c r="C215" t="n">
-        <v>11.62048109847782</v>
+        <v>11.62048009790152</v>
       </c>
       <c r="D215" t="n">
-        <v>11.02798956545112</v>
+        <v>11.02798861589103</v>
       </c>
       <c r="E215" t="n">
-        <v>11.56314370796374</v>
+        <v>11.56314271232445</v>
       </c>
       <c r="F215" t="n">
         <v>15779400</v>
@@ -4792,16 +4792,16 @@
         <v>44573</v>
       </c>
       <c r="B219" t="n">
-        <v>11.27645301818848</v>
+        <v>11.27645206451416</v>
       </c>
       <c r="C219" t="n">
-        <v>11.28600955287783</v>
+        <v>11.2860085983953</v>
       </c>
       <c r="D219" t="n">
-        <v>10.80819375474579</v>
+        <v>10.80819284067318</v>
       </c>
       <c r="E219" t="n">
-        <v>10.94198159495152</v>
+        <v>10.94198066956419</v>
       </c>
       <c r="F219" t="n">
         <v>7862000</v>
@@ -4812,16 +4812,16 @@
         <v>44574</v>
       </c>
       <c r="B220" t="n">
-        <v>11.48669242858887</v>
+        <v>11.48669338226318</v>
       </c>
       <c r="C220" t="n">
-        <v>11.57269850823688</v>
+        <v>11.57269946905179</v>
       </c>
       <c r="D220" t="n">
-        <v>11.15222099941061</v>
+        <v>11.15222192531568</v>
       </c>
       <c r="E220" t="n">
-        <v>11.27645321849507</v>
+        <v>11.27645415471443</v>
       </c>
       <c r="F220" t="n">
         <v>9668300</v>
@@ -4852,16 +4852,16 @@
         <v>44578</v>
       </c>
       <c r="B222" t="n">
-        <v>11.47713661193848</v>
+        <v>11.47713565826416</v>
       </c>
       <c r="C222" t="n">
-        <v>11.61092446289281</v>
+        <v>11.6109234981016</v>
       </c>
       <c r="D222" t="n">
-        <v>11.41024177509993</v>
+        <v>11.41024082698413</v>
       </c>
       <c r="E222" t="n">
-        <v>11.59181230333992</v>
+        <v>11.59181134013681</v>
       </c>
       <c r="F222" t="n">
         <v>4569300</v>
@@ -4912,16 +4912,16 @@
         <v>44581</v>
       </c>
       <c r="B225" t="n">
-        <v>11.41979694366455</v>
+        <v>11.41979789733887</v>
       </c>
       <c r="C225" t="n">
-        <v>11.69693005922028</v>
+        <v>11.69693103603816</v>
       </c>
       <c r="D225" t="n">
-        <v>11.36245956050752</v>
+        <v>11.36246050939355</v>
       </c>
       <c r="E225" t="n">
-        <v>11.56314222427969</v>
+        <v>11.56314318992485</v>
       </c>
       <c r="F225" t="n">
         <v>7365800</v>
@@ -4932,16 +4932,16 @@
         <v>44582</v>
       </c>
       <c r="B226" t="n">
-        <v>11.48669242858887</v>
+        <v>11.48669338226318</v>
       </c>
       <c r="C226" t="n">
-        <v>11.63003680603022</v>
+        <v>11.6300377716056</v>
       </c>
       <c r="D226" t="n">
-        <v>11.21911492070173</v>
+        <v>11.21911585216062</v>
       </c>
       <c r="E226" t="n">
-        <v>11.37201583300219</v>
+        <v>11.37201677715557</v>
       </c>
       <c r="F226" t="n">
         <v>8537100</v>
@@ -5012,16 +5012,16 @@
         <v>44588</v>
       </c>
       <c r="B230" t="n">
-        <v>11.99317741394043</v>
+        <v>11.99317646026611</v>
       </c>
       <c r="C230" t="n">
-        <v>12.13652179718475</v>
+        <v>12.13652083211196</v>
       </c>
       <c r="D230" t="n">
-        <v>11.66826250646786</v>
+        <v>11.66826157863015</v>
       </c>
       <c r="E230" t="n">
-        <v>11.85938865458074</v>
+        <v>11.85938771154504</v>
       </c>
       <c r="F230" t="n">
         <v>13761300</v>
@@ -5032,16 +5032,16 @@
         <v>44589</v>
       </c>
       <c r="B231" t="n">
-        <v>11.83071994781494</v>
+        <v>11.83071804046631</v>
       </c>
       <c r="C231" t="n">
-        <v>12.04095916619962</v>
+        <v>12.04095722495622</v>
       </c>
       <c r="D231" t="n">
-        <v>11.4580232758641</v>
+        <v>11.45802142860162</v>
       </c>
       <c r="E231" t="n">
-        <v>11.94539563656258</v>
+        <v>11.94539371072593</v>
       </c>
       <c r="F231" t="n">
         <v>14924100</v>
@@ -5052,16 +5052,16 @@
         <v>44592</v>
       </c>
       <c r="B232" t="n">
-        <v>11.97406387329102</v>
+        <v>11.97406482696533</v>
       </c>
       <c r="C232" t="n">
-        <v>12.12696478577772</v>
+        <v>12.12696575162983</v>
       </c>
       <c r="D232" t="n">
-        <v>11.76382557430247</v>
+        <v>11.76382651123235</v>
       </c>
       <c r="E232" t="n">
-        <v>11.81160642593357</v>
+        <v>11.81160736666896</v>
       </c>
       <c r="F232" t="n">
         <v>12073700</v>
@@ -5092,16 +5092,16 @@
         <v>44594</v>
       </c>
       <c r="B234" t="n">
-        <v>11.94539642333984</v>
+        <v>11.94539546966553</v>
       </c>
       <c r="C234" t="n">
-        <v>12.27986788773793</v>
+        <v>12.2798669073607</v>
       </c>
       <c r="D234" t="n">
-        <v>11.81160765530833</v>
+        <v>11.81160671231519</v>
       </c>
       <c r="E234" t="n">
-        <v>12.0218468875403</v>
+        <v>12.02184592776248</v>
       </c>
       <c r="F234" t="n">
         <v>9442200</v>
@@ -5112,16 +5112,16 @@
         <v>44595</v>
       </c>
       <c r="B235" t="n">
-        <v>11.94539642333984</v>
+        <v>11.94539546966553</v>
       </c>
       <c r="C235" t="n">
-        <v>12.21297304804146</v>
+        <v>12.21297207300486</v>
       </c>
       <c r="D235" t="n">
-        <v>11.8976146553742</v>
+        <v>11.8976137055146</v>
       </c>
       <c r="E235" t="n">
-        <v>12.04095995927113</v>
+        <v>12.04095899796739</v>
       </c>
       <c r="F235" t="n">
         <v>8796800</v>
@@ -5152,16 +5152,16 @@
         <v>44599</v>
       </c>
       <c r="B237" t="n">
-        <v>12.2034158706665</v>
+        <v>12.20341682434082</v>
       </c>
       <c r="C237" t="n">
-        <v>12.60478030096504</v>
+        <v>12.60478128600524</v>
       </c>
       <c r="D237" t="n">
-        <v>12.2034158706665</v>
+        <v>12.20341682434082</v>
       </c>
       <c r="E237" t="n">
-        <v>12.29897848307614</v>
+        <v>12.29897944421849</v>
       </c>
       <c r="F237" t="n">
         <v>7212000</v>
@@ -5192,16 +5192,16 @@
         <v>44601</v>
       </c>
       <c r="B239" t="n">
-        <v>12.05051326751709</v>
+        <v>12.05051517486572</v>
       </c>
       <c r="C239" t="n">
-        <v>12.28942115006283</v>
+        <v>12.28942309522567</v>
       </c>
       <c r="D239" t="n">
-        <v>11.91672543656267</v>
+        <v>11.91672732273544</v>
       </c>
       <c r="E239" t="n">
-        <v>11.95495066131554</v>
+        <v>11.95495255353858</v>
       </c>
       <c r="F239" t="n">
         <v>9060800</v>
@@ -5212,16 +5212,16 @@
         <v>44602</v>
       </c>
       <c r="B240" t="n">
-        <v>12.11740970611572</v>
+        <v>12.11740875244141</v>
       </c>
       <c r="C240" t="n">
-        <v>12.29897932000246</v>
+        <v>12.29897835203811</v>
       </c>
       <c r="D240" t="n">
-        <v>11.88805741573067</v>
+        <v>11.88805648010703</v>
       </c>
       <c r="E240" t="n">
-        <v>11.95495225146694</v>
+        <v>11.95495131057848</v>
       </c>
       <c r="F240" t="n">
         <v>4310600</v>
@@ -5232,16 +5232,16 @@
         <v>44603</v>
       </c>
       <c r="B241" t="n">
-        <v>11.79249382019043</v>
+        <v>11.79249286651611</v>
       </c>
       <c r="C241" t="n">
-        <v>12.21297131357752</v>
+        <v>12.21297032589864</v>
       </c>
       <c r="D241" t="n">
-        <v>11.74471205901066</v>
+        <v>11.74471110920052</v>
       </c>
       <c r="E241" t="n">
-        <v>12.18430262141418</v>
+        <v>12.18430163605377</v>
       </c>
       <c r="F241" t="n">
         <v>7316000</v>
@@ -5252,16 +5252,16 @@
         <v>44606</v>
       </c>
       <c r="B242" t="n">
-        <v>11.78293895721436</v>
+        <v>11.78293800354004</v>
       </c>
       <c r="C242" t="n">
-        <v>11.97406511768535</v>
+        <v>11.97406414854188</v>
       </c>
       <c r="D242" t="n">
-        <v>11.63959456470146</v>
+        <v>11.639593622629</v>
       </c>
       <c r="E242" t="n">
-        <v>11.79249549307826</v>
+        <v>11.79249453863047</v>
       </c>
       <c r="F242" t="n">
         <v>5445000</v>
@@ -5272,16 +5272,16 @@
         <v>44607</v>
       </c>
       <c r="B243" t="n">
-        <v>11.63959312438965</v>
+        <v>11.63959407806396</v>
       </c>
       <c r="C243" t="n">
-        <v>11.95495147798393</v>
+        <v>11.95495245749671</v>
       </c>
       <c r="D243" t="n">
-        <v>11.53447306561735</v>
+        <v>11.5344740106788</v>
       </c>
       <c r="E243" t="n">
-        <v>11.92628187393986</v>
+        <v>11.92628285110363</v>
       </c>
       <c r="F243" t="n">
         <v>11329100</v>
@@ -5392,16 +5392,16 @@
         <v>44615</v>
       </c>
       <c r="B249" t="n">
-        <v>12.73856830596924</v>
+        <v>12.73856925964355</v>
       </c>
       <c r="C249" t="n">
-        <v>12.87235704914128</v>
+        <v>12.87235801283171</v>
       </c>
       <c r="D249" t="n">
-        <v>12.51877349007365</v>
+        <v>12.51877442729301</v>
       </c>
       <c r="E249" t="n">
-        <v>12.51877349007365</v>
+        <v>12.51877442729301</v>
       </c>
       <c r="F249" t="n">
         <v>5598100</v>
@@ -5432,16 +5432,16 @@
         <v>44617</v>
       </c>
       <c r="B251" t="n">
-        <v>12.86280155181885</v>
+        <v>12.86280059814453</v>
       </c>
       <c r="C251" t="n">
-        <v>13.13993468322886</v>
+        <v>13.13993370900733</v>
       </c>
       <c r="D251" t="n">
-        <v>12.72901279786317</v>
+        <v>12.72901185410822</v>
       </c>
       <c r="E251" t="n">
-        <v>12.83413285860025</v>
+        <v>12.83413190705149</v>
       </c>
       <c r="F251" t="n">
         <v>8089600</v>
@@ -5472,16 +5472,16 @@
         <v>44623</v>
       </c>
       <c r="B253" t="n">
-        <v>12.56655502319336</v>
+        <v>12.56655597686768</v>
       </c>
       <c r="C253" t="n">
-        <v>12.95836473998952</v>
+        <v>12.95836572339823</v>
       </c>
       <c r="D253" t="n">
-        <v>12.337203660699</v>
+        <v>12.33720459696787</v>
       </c>
       <c r="E253" t="n">
-        <v>12.80546292029864</v>
+        <v>12.80546389210365</v>
       </c>
       <c r="F253" t="n">
         <v>12631200</v>
@@ -5492,16 +5492,16 @@
         <v>44624</v>
       </c>
       <c r="B254" t="n">
-        <v>12.14607810974121</v>
+        <v>12.14607715606689</v>
       </c>
       <c r="C254" t="n">
-        <v>12.64300608572388</v>
+        <v>12.64300509303224</v>
       </c>
       <c r="D254" t="n">
-        <v>12.13652157467044</v>
+        <v>12.13652062174647</v>
       </c>
       <c r="E254" t="n">
-        <v>12.64300608572388</v>
+        <v>12.64300509303224</v>
       </c>
       <c r="F254" t="n">
         <v>6563400</v>
@@ -5572,16 +5572,16 @@
         <v>44630</v>
       </c>
       <c r="B258" t="n">
-        <v>12.71945667266846</v>
+        <v>12.71945762634277</v>
       </c>
       <c r="C258" t="n">
-        <v>13.02525848523527</v>
+        <v>13.02525946183787</v>
       </c>
       <c r="D258" t="n">
-        <v>12.24164088485217</v>
+        <v>12.24164180270101</v>
       </c>
       <c r="E258" t="n">
-        <v>12.67167491161457</v>
+        <v>12.67167586170632</v>
       </c>
       <c r="F258" t="n">
         <v>9185900</v>
@@ -5592,16 +5592,16 @@
         <v>44631</v>
       </c>
       <c r="B259" t="n">
-        <v>12.40409755706787</v>
+        <v>12.40409851074219</v>
       </c>
       <c r="C259" t="n">
-        <v>12.92969511198934</v>
+        <v>12.9296961060736</v>
       </c>
       <c r="D259" t="n">
-        <v>12.20341579878139</v>
+        <v>12.20341673702652</v>
       </c>
       <c r="E259" t="n">
-        <v>12.92969511198934</v>
+        <v>12.9296961060736</v>
       </c>
       <c r="F259" t="n">
         <v>7293900</v>
@@ -5632,16 +5632,16 @@
         <v>44635</v>
       </c>
       <c r="B261" t="n">
-        <v>12.82457637786865</v>
+        <v>12.82457542419434</v>
       </c>
       <c r="C261" t="n">
-        <v>12.90102683434848</v>
+        <v>12.90102587498907</v>
       </c>
       <c r="D261" t="n">
-        <v>12.29897880604886</v>
+        <v>12.29897789145957</v>
       </c>
       <c r="E261" t="n">
-        <v>12.29897880604886</v>
+        <v>12.29897789145957</v>
       </c>
       <c r="F261" t="n">
         <v>8181800</v>
@@ -5652,16 +5652,16 @@
         <v>44636</v>
       </c>
       <c r="B262" t="n">
-        <v>12.99658966064453</v>
+        <v>12.99659061431885</v>
       </c>
       <c r="C262" t="n">
-        <v>13.09215227041673</v>
+        <v>13.09215323110332</v>
       </c>
       <c r="D262" t="n">
-        <v>12.7385687004009</v>
+        <v>12.73856963514194</v>
       </c>
       <c r="E262" t="n">
-        <v>12.91058267389665</v>
+        <v>12.91058362125988</v>
       </c>
       <c r="F262" t="n">
         <v>7731200</v>
@@ -5692,16 +5692,16 @@
         <v>44638</v>
       </c>
       <c r="B264" t="n">
-        <v>13.58908271789551</v>
+        <v>13.58908176422119</v>
       </c>
       <c r="C264" t="n">
-        <v>13.78020887124509</v>
+        <v>13.78020790415765</v>
       </c>
       <c r="D264" t="n">
-        <v>12.98703465132328</v>
+        <v>12.98703373990036</v>
       </c>
       <c r="E264" t="n">
-        <v>13.04437204164746</v>
+        <v>13.04437112620064</v>
       </c>
       <c r="F264" t="n">
         <v>10366600</v>
@@ -5732,16 +5732,16 @@
         <v>44642</v>
       </c>
       <c r="B266" t="n">
-        <v>14.08601093292236</v>
+        <v>14.08600997924805</v>
       </c>
       <c r="C266" t="n">
-        <v>14.26758146491387</v>
+        <v>14.26758049894657</v>
       </c>
       <c r="D266" t="n">
-        <v>13.62730815783909</v>
+        <v>13.62730723522063</v>
       </c>
       <c r="E266" t="n">
-        <v>13.66553338909603</v>
+        <v>13.66553246388958</v>
       </c>
       <c r="F266" t="n">
         <v>13737200</v>
@@ -5792,16 +5792,16 @@
         <v>44645</v>
       </c>
       <c r="B269" t="n">
-        <v>15.13720607757568</v>
+        <v>15.13720512390137</v>
       </c>
       <c r="C269" t="n">
-        <v>15.24232523512279</v>
+        <v>15.24232427482575</v>
       </c>
       <c r="D269" t="n">
-        <v>14.64027716256451</v>
+        <v>14.64027624019771</v>
       </c>
       <c r="E269" t="n">
-        <v>14.71672762466447</v>
+        <v>14.71672669748114</v>
       </c>
       <c r="F269" t="n">
         <v>8426200</v>
@@ -5812,16 +5812,16 @@
         <v>44648</v>
       </c>
       <c r="B270" t="n">
-        <v>15.51945686340332</v>
+        <v>15.51945781707764</v>
       </c>
       <c r="C270" t="n">
-        <v>15.7774778311631</v>
+        <v>15.77747880069286</v>
       </c>
       <c r="D270" t="n">
-        <v>14.97474714661442</v>
+        <v>14.9747480668162</v>
       </c>
       <c r="E270" t="n">
-        <v>15.19454197571826</v>
+        <v>15.19454290942648</v>
       </c>
       <c r="F270" t="n">
         <v>14496800</v>
@@ -5852,16 +5852,16 @@
         <v>44650</v>
       </c>
       <c r="B272" t="n">
-        <v>15.45256423950195</v>
+        <v>15.45256519317627</v>
       </c>
       <c r="C272" t="n">
-        <v>15.82526000904275</v>
+        <v>15.82526098571845</v>
       </c>
       <c r="D272" t="n">
-        <v>15.3952268494317</v>
+        <v>15.39522779956737</v>
       </c>
       <c r="E272" t="n">
-        <v>15.51945816503771</v>
+        <v>15.51945912284047</v>
       </c>
       <c r="F272" t="n">
         <v>8944100</v>
@@ -5872,16 +5872,16 @@
         <v>44651</v>
       </c>
       <c r="B273" t="n">
-        <v>15.56723976135254</v>
+        <v>15.56724071502686</v>
       </c>
       <c r="C273" t="n">
-        <v>15.81570237531094</v>
+        <v>15.81570334420647</v>
       </c>
       <c r="D273" t="n">
-        <v>15.42389356204693</v>
+        <v>15.42389450693963</v>
       </c>
       <c r="E273" t="n">
-        <v>15.42389356204693</v>
+        <v>15.42389450693963</v>
       </c>
       <c r="F273" t="n">
         <v>17319900</v>
@@ -5892,16 +5892,16 @@
         <v>44652</v>
       </c>
       <c r="B274" t="n">
-        <v>15.74880886077881</v>
+        <v>15.74880695343018</v>
       </c>
       <c r="C274" t="n">
-        <v>15.97816023377391</v>
+        <v>15.97815829864838</v>
       </c>
       <c r="D274" t="n">
-        <v>15.47167663526406</v>
+        <v>15.4716747614791</v>
       </c>
       <c r="E274" t="n">
-        <v>15.7201410783561</v>
+        <v>15.72013917447944</v>
       </c>
       <c r="F274" t="n">
         <v>8302400</v>
@@ -5912,16 +5912,16 @@
         <v>44655</v>
       </c>
       <c r="B275" t="n">
-        <v>15.56723976135254</v>
+        <v>15.56724071502686</v>
       </c>
       <c r="C275" t="n">
-        <v>15.86348504932035</v>
+        <v>15.86348602114313</v>
       </c>
       <c r="D275" t="n">
-        <v>15.52901362214501</v>
+        <v>15.52901457347753</v>
       </c>
       <c r="E275" t="n">
-        <v>15.75836498922228</v>
+        <v>15.75836595460524</v>
       </c>
       <c r="F275" t="n">
         <v>2672100</v>
@@ -5932,16 +5932,16 @@
         <v>44656</v>
       </c>
       <c r="B276" t="n">
-        <v>15.45256423950195</v>
+        <v>15.45256519317627</v>
       </c>
       <c r="C276" t="n">
-        <v>15.65324601610922</v>
+        <v>15.65324698216886</v>
       </c>
       <c r="D276" t="n">
-        <v>15.35700070756969</v>
+        <v>15.35700165534618</v>
       </c>
       <c r="E276" t="n">
-        <v>15.57679555510796</v>
+        <v>15.57679651644937</v>
       </c>
       <c r="F276" t="n">
         <v>10716200</v>
@@ -5952,16 +5952,16 @@
         <v>44657</v>
       </c>
       <c r="B277" t="n">
-        <v>15.56723976135254</v>
+        <v>15.56724071502686</v>
       </c>
       <c r="C277" t="n">
-        <v>15.70102760313362</v>
+        <v>15.701028565004</v>
       </c>
       <c r="D277" t="n">
-        <v>15.13720480888101</v>
+        <v>15.13720573621069</v>
       </c>
       <c r="E277" t="n">
-        <v>15.38566924556204</v>
+        <v>15.38567018811306</v>
       </c>
       <c r="F277" t="n">
         <v>10924400</v>
@@ -5972,16 +5972,16 @@
         <v>44658</v>
       </c>
       <c r="B278" t="n">
-        <v>15.38567066192627</v>
+        <v>15.38566875457764</v>
       </c>
       <c r="C278" t="n">
-        <v>15.52901505170514</v>
+        <v>15.52901312658622</v>
       </c>
       <c r="D278" t="n">
-        <v>15.25188189646763</v>
+        <v>15.25188000570468</v>
       </c>
       <c r="E278" t="n">
-        <v>15.366557590563</v>
+        <v>15.3665556855838</v>
       </c>
       <c r="F278" t="n">
         <v>6566700</v>
@@ -5992,16 +5992,16 @@
         <v>44659</v>
       </c>
       <c r="B279" t="n">
-        <v>15.40478229522705</v>
+        <v>15.40478324890137</v>
       </c>
       <c r="C279" t="n">
-        <v>15.57679445327038</v>
+        <v>15.57679541759357</v>
       </c>
       <c r="D279" t="n">
-        <v>15.07031086848462</v>
+        <v>15.07031180145259</v>
       </c>
       <c r="E279" t="n">
-        <v>15.32833183963358</v>
+        <v>15.32833278857503</v>
       </c>
       <c r="F279" t="n">
         <v>3069100</v>
@@ -6012,16 +6012,16 @@
         <v>44662</v>
       </c>
       <c r="B280" t="n">
-        <v>15.29010677337646</v>
+        <v>15.29010581970215</v>
       </c>
       <c r="C280" t="n">
-        <v>15.4907885498701</v>
+        <v>15.49078758367887</v>
       </c>
       <c r="D280" t="n">
-        <v>15.21365631241849</v>
+        <v>15.21365536351254</v>
       </c>
       <c r="E280" t="n">
-        <v>15.38567030525462</v>
+        <v>15.38566934561982</v>
       </c>
       <c r="F280" t="n">
         <v>10289300</v>
@@ -6032,16 +6032,16 @@
         <v>44663</v>
       </c>
       <c r="B281" t="n">
-        <v>15.72013854980469</v>
+        <v>15.72014236450195</v>
       </c>
       <c r="C281" t="n">
-        <v>15.82525677298439</v>
+        <v>15.82526061318996</v>
       </c>
       <c r="D281" t="n">
-        <v>15.39522370130949</v>
+        <v>15.39522743716192</v>
       </c>
       <c r="E281" t="n">
-        <v>15.48123068018895</v>
+        <v>15.48123443691209</v>
       </c>
       <c r="F281" t="n">
         <v>9798400</v>
@@ -6112,16 +6112,16 @@
         <v>44670</v>
       </c>
       <c r="B285" t="n">
-        <v>15.61502075195312</v>
+        <v>15.61502265930176</v>
       </c>
       <c r="C285" t="n">
-        <v>15.77747819958926</v>
+        <v>15.7774801267818</v>
       </c>
       <c r="D285" t="n">
-        <v>15.18498670700624</v>
+        <v>15.18498856182694</v>
       </c>
       <c r="E285" t="n">
-        <v>15.32833199622942</v>
+        <v>15.3283338685595</v>
       </c>
       <c r="F285" t="n">
         <v>7756800</v>
@@ -6132,16 +6132,16 @@
         <v>44671</v>
       </c>
       <c r="B286" t="n">
-        <v>15.853928565979</v>
+        <v>15.85393047332764</v>
       </c>
       <c r="C286" t="n">
-        <v>16.33174437128826</v>
+        <v>16.33174633612178</v>
       </c>
       <c r="D286" t="n">
-        <v>15.72014072376366</v>
+        <v>15.72014261501659</v>
       </c>
       <c r="E286" t="n">
-        <v>15.74880850553972</v>
+        <v>15.74881040024161</v>
       </c>
       <c r="F286" t="n">
         <v>12326800</v>
@@ -6172,16 +6172,16 @@
         <v>44676</v>
       </c>
       <c r="B288" t="n">
-        <v>15.29966163635254</v>
+        <v>15.29966259002686</v>
       </c>
       <c r="C288" t="n">
-        <v>15.46211907596952</v>
+        <v>15.4621200397703</v>
       </c>
       <c r="D288" t="n">
-        <v>15.01297198341896</v>
+        <v>15.01297291922304</v>
       </c>
       <c r="E288" t="n">
-        <v>15.2805485675217</v>
+        <v>15.28054952000464</v>
       </c>
       <c r="F288" t="n">
         <v>6454900</v>
@@ -6212,16 +6212,16 @@
         <v>44678</v>
       </c>
       <c r="B290" t="n">
-        <v>15.18498802185059</v>
+        <v>15.18498706817627</v>
       </c>
       <c r="C290" t="n">
-        <v>15.48123424947426</v>
+        <v>15.48123327719457</v>
       </c>
       <c r="D290" t="n">
-        <v>14.96519225722114</v>
+        <v>14.96519131735082</v>
       </c>
       <c r="E290" t="n">
-        <v>15.29010718062729</v>
+        <v>15.2901062203511</v>
       </c>
       <c r="F290" t="n">
         <v>7959000</v>
@@ -6252,16 +6252,16 @@
         <v>44680</v>
       </c>
       <c r="B292" t="n">
-        <v>14.72057151794434</v>
+        <v>14.72057247161865</v>
       </c>
       <c r="C292" t="n">
-        <v>15.13482874017579</v>
+        <v>15.13482972068782</v>
       </c>
       <c r="D292" t="n">
-        <v>14.72057151794434</v>
+        <v>14.72057247161865</v>
       </c>
       <c r="E292" t="n">
-        <v>15.06739185981573</v>
+        <v>15.06739283595885</v>
       </c>
       <c r="F292" t="n">
         <v>7651000</v>
@@ -6292,16 +6292,16 @@
         <v>44684</v>
       </c>
       <c r="B294" t="n">
-        <v>14.62423515319824</v>
+        <v>14.62423324584961</v>
       </c>
       <c r="C294" t="n">
-        <v>14.85544813205102</v>
+        <v>14.85544619454671</v>
       </c>
       <c r="D294" t="n">
-        <v>14.47972635234622</v>
+        <v>14.47972446384498</v>
       </c>
       <c r="E294" t="n">
-        <v>14.70130614614917</v>
+        <v>14.70130422874864</v>
       </c>
       <c r="F294" t="n">
         <v>5388000</v>
@@ -6312,16 +6312,16 @@
         <v>44685</v>
       </c>
       <c r="B295" t="n">
-        <v>14.79764175415039</v>
+        <v>14.79764270782471</v>
       </c>
       <c r="C295" t="n">
-        <v>14.95178463095864</v>
+        <v>14.95178559456712</v>
       </c>
       <c r="D295" t="n">
-        <v>14.2581449009764</v>
+        <v>14.25814581988137</v>
       </c>
       <c r="E295" t="n">
-        <v>14.43155414440306</v>
+        <v>14.43155507448386</v>
       </c>
       <c r="F295" t="n">
         <v>5127000</v>
@@ -6352,16 +6352,16 @@
         <v>44687</v>
       </c>
       <c r="B297" t="n">
-        <v>14.15217208862305</v>
+        <v>14.15217304229736</v>
       </c>
       <c r="C297" t="n">
-        <v>14.51825971060268</v>
+        <v>14.51826068894659</v>
       </c>
       <c r="D297" t="n">
-        <v>14.05583382100224</v>
+        <v>14.0558347681846</v>
       </c>
       <c r="E297" t="n">
-        <v>14.45082283139226</v>
+        <v>14.45082380519179</v>
       </c>
       <c r="F297" t="n">
         <v>6832100</v>
@@ -6372,16 +6372,16 @@
         <v>44690</v>
       </c>
       <c r="B298" t="n">
-        <v>14.21961116790771</v>
+        <v>14.2196102142334</v>
       </c>
       <c r="C298" t="n">
-        <v>14.32558354746724</v>
+        <v>14.32558258668562</v>
       </c>
       <c r="D298" t="n">
-        <v>13.92096039822737</v>
+        <v>13.92095946458282</v>
       </c>
       <c r="E298" t="n">
-        <v>14.04620098430244</v>
+        <v>14.04620004225831</v>
       </c>
       <c r="F298" t="n">
         <v>11844800</v>
@@ -6412,16 +6412,16 @@
         <v>44692</v>
       </c>
       <c r="B300" t="n">
-        <v>14.60496616363525</v>
+        <v>14.60496520996094</v>
       </c>
       <c r="C300" t="n">
-        <v>14.7880104511626</v>
+        <v>14.78800948553586</v>
       </c>
       <c r="D300" t="n">
-        <v>14.4026545882811</v>
+        <v>14.40265364781732</v>
       </c>
       <c r="E300" t="n">
-        <v>14.45082418598612</v>
+        <v>14.45082324237696</v>
       </c>
       <c r="F300" t="n">
         <v>6181500</v>
@@ -6492,16 +6492,16 @@
         <v>44698</v>
       </c>
       <c r="B304" t="n">
-        <v>15.25043678283691</v>
+        <v>15.2504358291626</v>
       </c>
       <c r="C304" t="n">
-        <v>15.26970498992616</v>
+        <v>15.26970403504692</v>
       </c>
       <c r="D304" t="n">
-        <v>14.84581362154963</v>
+        <v>14.84581269317811</v>
       </c>
       <c r="E304" t="n">
-        <v>14.84581362154963</v>
+        <v>14.84581269317811</v>
       </c>
       <c r="F304" t="n">
         <v>7407200</v>
@@ -6512,16 +6512,16 @@
         <v>44699</v>
       </c>
       <c r="B305" t="n">
-        <v>14.83617782592773</v>
+        <v>14.83617877960205</v>
       </c>
       <c r="C305" t="n">
-        <v>15.2504350435133</v>
+        <v>15.2504360238162</v>
       </c>
       <c r="D305" t="n">
-        <v>14.81691053979462</v>
+        <v>14.81691149223043</v>
       </c>
       <c r="E305" t="n">
-        <v>15.23116775738018</v>
+        <v>15.23116873644458</v>
       </c>
       <c r="F305" t="n">
         <v>6842800</v>
@@ -6532,16 +6532,16 @@
         <v>44700</v>
       </c>
       <c r="B306" t="n">
-        <v>14.88434791564941</v>
+        <v>14.88434886932373</v>
       </c>
       <c r="C306" t="n">
-        <v>14.95178571626016</v>
+        <v>14.95178667425537</v>
       </c>
       <c r="D306" t="n">
-        <v>14.6627690645589</v>
+        <v>14.66277000403615</v>
       </c>
       <c r="E306" t="n">
-        <v>14.92288340795901</v>
+        <v>14.92288436410238</v>
       </c>
       <c r="F306" t="n">
         <v>6219800</v>
@@ -6632,16 +6632,16 @@
         <v>44707</v>
       </c>
       <c r="B311" t="n">
-        <v>15.50091648101807</v>
+        <v>15.5009183883667</v>
       </c>
       <c r="C311" t="n">
-        <v>15.60688977236364</v>
+        <v>15.60689169275202</v>
       </c>
       <c r="D311" t="n">
-        <v>15.03848966141599</v>
+        <v>15.03849151186417</v>
       </c>
       <c r="E311" t="n">
-        <v>15.07702515315295</v>
+        <v>15.07702700834282</v>
       </c>
       <c r="F311" t="n">
         <v>6641000</v>
@@ -6672,16 +6672,16 @@
         <v>44711</v>
       </c>
       <c r="B313" t="n">
-        <v>15.26970481872559</v>
+        <v>15.26970386505127</v>
       </c>
       <c r="C313" t="n">
-        <v>15.4912836852155</v>
+        <v>15.4912827177024</v>
       </c>
       <c r="D313" t="n">
-        <v>15.16373151844026</v>
+        <v>15.16373057138454</v>
       </c>
       <c r="E313" t="n">
-        <v>15.23116932373783</v>
+        <v>15.23116837247026</v>
       </c>
       <c r="F313" t="n">
         <v>1706700</v>
@@ -6692,16 +6692,16 @@
         <v>44712</v>
       </c>
       <c r="B314" t="n">
-        <v>15.26006984710693</v>
+        <v>15.26007080078125</v>
       </c>
       <c r="C314" t="n">
-        <v>15.39494361251144</v>
+        <v>15.39494457461466</v>
       </c>
       <c r="D314" t="n">
-        <v>15.05775828024155</v>
+        <v>15.05775922127246</v>
       </c>
       <c r="E314" t="n">
-        <v>15.29860533990231</v>
+        <v>15.29860629598489</v>
       </c>
       <c r="F314" t="n">
         <v>5708500</v>
@@ -6712,16 +6712,16 @@
         <v>44713</v>
       </c>
       <c r="B315" t="n">
-        <v>14.85544586181641</v>
+        <v>14.85544681549072</v>
       </c>
       <c r="C315" t="n">
-        <v>15.53945059003543</v>
+        <v>15.53945158762076</v>
       </c>
       <c r="D315" t="n">
-        <v>14.73020528772095</v>
+        <v>14.73020623335521</v>
       </c>
       <c r="E315" t="n">
-        <v>15.39494273002606</v>
+        <v>15.39494371833443</v>
       </c>
       <c r="F315" t="n">
         <v>6096700</v>
@@ -6752,16 +6752,16 @@
         <v>44715</v>
       </c>
       <c r="B317" t="n">
-        <v>14.88434791564941</v>
+        <v>14.88434886932373</v>
       </c>
       <c r="C317" t="n">
-        <v>15.23116826519437</v>
+        <v>15.23116924109026</v>
       </c>
       <c r="D317" t="n">
-        <v>14.78800964425473</v>
+        <v>14.78801059175644</v>
       </c>
       <c r="E317" t="n">
-        <v>15.17336456735067</v>
+        <v>15.17336553954295</v>
       </c>
       <c r="F317" t="n">
         <v>4184100</v>
@@ -6792,16 +6792,16 @@
         <v>44719</v>
       </c>
       <c r="B319" t="n">
-        <v>15.12519454956055</v>
+        <v>15.12519550323486</v>
       </c>
       <c r="C319" t="n">
-        <v>15.31787200572364</v>
+        <v>15.31787297154666</v>
       </c>
       <c r="D319" t="n">
-        <v>14.70130414600175</v>
+        <v>14.70130507294891</v>
       </c>
       <c r="E319" t="n">
-        <v>14.8265447221974</v>
+        <v>14.82654565704124</v>
       </c>
       <c r="F319" t="n">
         <v>7316900</v>
@@ -6812,16 +6812,16 @@
         <v>44720</v>
       </c>
       <c r="B320" t="n">
-        <v>15.35640907287598</v>
+        <v>15.35640811920166</v>
       </c>
       <c r="C320" t="n">
-        <v>15.74176494350709</v>
+        <v>15.74176396590114</v>
       </c>
       <c r="D320" t="n">
-        <v>14.9903223279765</v>
+        <v>14.99032139703716</v>
       </c>
       <c r="E320" t="n">
-        <v>15.00958961619079</v>
+        <v>15.00958868405489</v>
       </c>
       <c r="F320" t="n">
         <v>10420600</v>
@@ -6832,16 +6832,16 @@
         <v>44721</v>
       </c>
       <c r="B321" t="n">
-        <v>15.02885723114014</v>
+        <v>15.02885627746582</v>
       </c>
       <c r="C321" t="n">
-        <v>15.50091725827793</v>
+        <v>15.50091627464848</v>
       </c>
       <c r="D321" t="n">
-        <v>14.76874195980382</v>
+        <v>14.76874102263543</v>
       </c>
       <c r="E321" t="n">
-        <v>15.38531077727023</v>
+        <v>15.38530980097672</v>
       </c>
       <c r="F321" t="n">
         <v>9688900</v>
@@ -6892,16 +6892,16 @@
         <v>44726</v>
       </c>
       <c r="B324" t="n">
-        <v>14.05583477020264</v>
+        <v>14.05583381652832</v>
       </c>
       <c r="C324" t="n">
-        <v>14.2099767438121</v>
+        <v>14.2099757796794</v>
       </c>
       <c r="D324" t="n">
-        <v>13.84388909711031</v>
+        <v>13.84388815781629</v>
       </c>
       <c r="E324" t="n">
-        <v>14.01729927680027</v>
+        <v>14.01729832574055</v>
       </c>
       <c r="F324" t="n">
         <v>10130900</v>
@@ -6932,16 +6932,16 @@
         <v>44729</v>
       </c>
       <c r="B326" t="n">
-        <v>14.94215202331543</v>
+        <v>14.94215297698975</v>
       </c>
       <c r="C326" t="n">
-        <v>15.18299908654582</v>
+        <v>15.18300005559206</v>
       </c>
       <c r="D326" t="n">
-        <v>14.56643027392291</v>
+        <v>14.56643120361701</v>
       </c>
       <c r="E326" t="n">
-        <v>14.63386715762466</v>
+        <v>14.63386809162287</v>
       </c>
       <c r="F326" t="n">
         <v>14099900</v>
@@ -6972,16 +6972,16 @@
         <v>44733</v>
       </c>
       <c r="B328" t="n">
-        <v>14.84581279754639</v>
+        <v>14.84581184387207</v>
       </c>
       <c r="C328" t="n">
-        <v>15.6454249721946</v>
+        <v>15.64542396715431</v>
       </c>
       <c r="D328" t="n">
-        <v>14.81691140727535</v>
+        <v>14.81691045545762</v>
       </c>
       <c r="E328" t="n">
-        <v>15.37567651922811</v>
+        <v>15.37567553151609</v>
       </c>
       <c r="F328" t="n">
         <v>9398400</v>
@@ -7012,16 +7012,16 @@
         <v>44735</v>
       </c>
       <c r="B330" t="n">
-        <v>14.72057151794434</v>
+        <v>14.72057247161865</v>
       </c>
       <c r="C330" t="n">
-        <v>14.90361579143392</v>
+        <v>14.90361675696679</v>
       </c>
       <c r="D330" t="n">
-        <v>14.39301938118073</v>
+        <v>14.39302031363454</v>
       </c>
       <c r="E330" t="n">
-        <v>14.39301938118073</v>
+        <v>14.39302031363454</v>
       </c>
       <c r="F330" t="n">
         <v>3851900</v>
@@ -7052,16 +7052,16 @@
         <v>44739</v>
       </c>
       <c r="B332" t="n">
-        <v>14.16180801391602</v>
+        <v>14.1618070602417</v>
       </c>
       <c r="C332" t="n">
-        <v>14.49899429088777</v>
+        <v>14.4989933145069</v>
       </c>
       <c r="D332" t="n">
-        <v>14.10400522965489</v>
+        <v>14.10400427987309</v>
       </c>
       <c r="E332" t="n">
-        <v>14.47972608362827</v>
+        <v>14.47972510854494</v>
       </c>
       <c r="F332" t="n">
         <v>8041800</v>
@@ -7152,16 +7152,16 @@
         <v>44746</v>
       </c>
       <c r="B337" t="n">
-        <v>13.8727912902832</v>
+        <v>13.87279033660889</v>
       </c>
       <c r="C337" t="n">
-        <v>14.14254067846864</v>
+        <v>14.14253970625061</v>
       </c>
       <c r="D337" t="n">
-        <v>13.76681890698379</v>
+        <v>13.76681796059447</v>
       </c>
       <c r="E337" t="n">
-        <v>13.95949638514576</v>
+        <v>13.95949542551097</v>
       </c>
       <c r="F337" t="n">
         <v>1980900</v>
@@ -7212,16 +7212,16 @@
         <v>44749</v>
       </c>
       <c r="B340" t="n">
-        <v>14.57606410980225</v>
+        <v>14.57606506347656</v>
       </c>
       <c r="C340" t="n">
-        <v>14.95178585230849</v>
+        <v>14.95178683056531</v>
       </c>
       <c r="D340" t="n">
-        <v>14.47009173467626</v>
+        <v>14.47009268141707</v>
       </c>
       <c r="E340" t="n">
-        <v>14.49899312448178</v>
+        <v>14.49899407311354</v>
       </c>
       <c r="F340" t="n">
         <v>6763400</v>
@@ -7232,16 +7232,16 @@
         <v>44750</v>
       </c>
       <c r="B341" t="n">
-        <v>14.72057151794434</v>
+        <v>14.72057247161865</v>
       </c>
       <c r="C341" t="n">
-        <v>14.82654480851997</v>
+        <v>14.82654576905978</v>
       </c>
       <c r="D341" t="n">
-        <v>14.41228758628851</v>
+        <v>14.41228851999061</v>
       </c>
       <c r="E341" t="n">
-        <v>14.73983972305212</v>
+        <v>14.73984067797473</v>
       </c>
       <c r="F341" t="n">
         <v>3792400</v>
@@ -7252,16 +7252,16 @@
         <v>44753</v>
       </c>
       <c r="B342" t="n">
-        <v>14.788010597229</v>
+        <v>14.78800964355469</v>
       </c>
       <c r="C342" t="n">
-        <v>14.89398297821984</v>
+        <v>14.8939820177114</v>
       </c>
       <c r="D342" t="n">
-        <v>14.52789531830785</v>
+        <v>14.52789438140829</v>
       </c>
       <c r="E342" t="n">
-        <v>14.57606491648865</v>
+        <v>14.57606397648265</v>
       </c>
       <c r="F342" t="n">
         <v>3654100</v>
@@ -7292,16 +7292,16 @@
         <v>44755</v>
       </c>
       <c r="B344" t="n">
-        <v>14.77837562561035</v>
+        <v>14.77837657928467</v>
       </c>
       <c r="C344" t="n">
-        <v>15.01922268360593</v>
+        <v>15.01922365282253</v>
       </c>
       <c r="D344" t="n">
-        <v>14.44118937691309</v>
+        <v>14.44119030882819</v>
       </c>
       <c r="E344" t="n">
-        <v>14.58569816296561</v>
+        <v>14.58569910420611</v>
       </c>
       <c r="F344" t="n">
         <v>3964800</v>
@@ -7392,16 +7392,16 @@
         <v>44762</v>
       </c>
       <c r="B349" t="n">
-        <v>14.82654571533203</v>
+        <v>14.82654476165771</v>
       </c>
       <c r="C349" t="n">
-        <v>15.10592827517219</v>
+        <v>15.10592730352741</v>
       </c>
       <c r="D349" t="n">
-        <v>14.57606454616261</v>
+        <v>14.57606360859976</v>
       </c>
       <c r="E349" t="n">
-        <v>14.89398259981663</v>
+        <v>14.89398164180463</v>
       </c>
       <c r="F349" t="n">
         <v>5599700</v>
@@ -7412,16 +7412,16 @@
         <v>44763</v>
       </c>
       <c r="B350" t="n">
-        <v>14.84581279754639</v>
+        <v>14.84581184387207</v>
       </c>
       <c r="C350" t="n">
-        <v>14.95178609313791</v>
+        <v>14.95178513265602</v>
       </c>
       <c r="D350" t="n">
-        <v>14.60496573485093</v>
+        <v>14.6049647966483</v>
       </c>
       <c r="E350" t="n">
-        <v>14.74947452372338</v>
+        <v>14.7494735762377</v>
       </c>
       <c r="F350" t="n">
         <v>4662200</v>
@@ -7492,16 +7492,16 @@
         <v>44769</v>
       </c>
       <c r="B354" t="n">
-        <v>15.76103115081787</v>
+        <v>15.7610330581665</v>
       </c>
       <c r="C354" t="n">
-        <v>15.9344413165386</v>
+        <v>15.93444324487276</v>
       </c>
       <c r="D354" t="n">
-        <v>15.03848909990104</v>
+        <v>15.03849091980999</v>
       </c>
       <c r="E354" t="n">
-        <v>15.04812320216521</v>
+        <v>15.04812502324004</v>
       </c>
       <c r="F354" t="n">
         <v>22102600</v>
@@ -7512,16 +7512,16 @@
         <v>44770</v>
       </c>
       <c r="B355" t="n">
-        <v>15.59725761413574</v>
+        <v>15.59725570678711</v>
       </c>
       <c r="C355" t="n">
-        <v>16.13675456570828</v>
+        <v>16.13675259238595</v>
       </c>
       <c r="D355" t="n">
-        <v>15.31787411576586</v>
+        <v>15.31787224258232</v>
       </c>
       <c r="E355" t="n">
-        <v>15.91517569028781</v>
+        <v>15.91517374406179</v>
       </c>
       <c r="F355" t="n">
         <v>25902000</v>
@@ -7532,16 +7532,16 @@
         <v>44771</v>
       </c>
       <c r="B356" t="n">
-        <v>15.26970481872559</v>
+        <v>15.26970386505127</v>
       </c>
       <c r="C356" t="n">
-        <v>15.66469387203972</v>
+        <v>15.66469289369624</v>
       </c>
       <c r="D356" t="n">
-        <v>15.26970481872559</v>
+        <v>15.26970386505127</v>
       </c>
       <c r="E356" t="n">
-        <v>15.59725698550082</v>
+        <v>15.59725601136913</v>
       </c>
       <c r="F356" t="n">
         <v>15825800</v>
@@ -7612,16 +7612,16 @@
         <v>44777</v>
       </c>
       <c r="B360" t="n">
-        <v>16.21382331848145</v>
+        <v>16.21382522583008</v>
       </c>
       <c r="C360" t="n">
-        <v>16.42576806079203</v>
+        <v>16.42576999307324</v>
       </c>
       <c r="D360" t="n">
-        <v>15.92480759373818</v>
+        <v>15.92480946708782</v>
       </c>
       <c r="E360" t="n">
-        <v>16.02114494364116</v>
+        <v>16.02114682832365</v>
       </c>
       <c r="F360" t="n">
         <v>10048700</v>
@@ -7692,16 +7692,16 @@
         <v>44783</v>
       </c>
       <c r="B364" t="n">
-        <v>16.89782905578613</v>
+        <v>16.89783096313477</v>
       </c>
       <c r="C364" t="n">
-        <v>17.20611297019896</v>
+        <v>17.20611491234526</v>
       </c>
       <c r="D364" t="n">
-        <v>16.73405299656468</v>
+        <v>16.73405488542704</v>
       </c>
       <c r="E364" t="n">
-        <v>17.16757656213882</v>
+        <v>17.1675784999353</v>
       </c>
       <c r="F364" t="n">
         <v>6533000</v>
@@ -7752,16 +7752,16 @@
         <v>44788</v>
       </c>
       <c r="B367" t="n">
-        <v>17.53366851806641</v>
+        <v>17.53366661071777</v>
       </c>
       <c r="C367" t="n">
-        <v>17.66854229762282</v>
+        <v>17.66854037560234</v>
       </c>
       <c r="D367" t="n">
-        <v>17.06160661458408</v>
+        <v>17.06160475858731</v>
       </c>
       <c r="E367" t="n">
-        <v>17.20611633555731</v>
+        <v>17.20611446384048</v>
       </c>
       <c r="F367" t="n">
         <v>7999500</v>
@@ -7772,16 +7772,16 @@
         <v>44789</v>
       </c>
       <c r="B368" t="n">
-        <v>17.42769432067871</v>
+        <v>17.42769241333008</v>
       </c>
       <c r="C368" t="n">
-        <v>17.63000497965835</v>
+        <v>17.63000305016812</v>
       </c>
       <c r="D368" t="n">
-        <v>17.19648135148026</v>
+        <v>17.1964794694364</v>
       </c>
       <c r="E368" t="n">
-        <v>17.52403351722407</v>
+        <v>17.52403159933173</v>
       </c>
       <c r="F368" t="n">
         <v>4828900</v>
@@ -7832,16 +7832,16 @@
         <v>44792</v>
       </c>
       <c r="B371" t="n">
-        <v>17.12904167175293</v>
+        <v>17.12904357910156</v>
       </c>
       <c r="C371" t="n">
-        <v>17.57219933106722</v>
+        <v>17.57220128776223</v>
       </c>
       <c r="D371" t="n">
-        <v>17.07123706074208</v>
+        <v>17.07123896165407</v>
       </c>
       <c r="E371" t="n">
-        <v>17.4565937840796</v>
+        <v>17.45659572790173</v>
       </c>
       <c r="F371" t="n">
         <v>7571900</v>
@@ -7852,16 +7852,16 @@
         <v>44795</v>
       </c>
       <c r="B372" t="n">
-        <v>17.36025619506836</v>
+        <v>17.36025810241699</v>
       </c>
       <c r="C372" t="n">
-        <v>17.45659538473642</v>
+        <v>17.45659730266971</v>
       </c>
       <c r="D372" t="n">
-        <v>16.82075746793411</v>
+        <v>16.82075931600872</v>
       </c>
       <c r="E372" t="n">
-        <v>16.98453353911465</v>
+        <v>16.98453540518312</v>
       </c>
       <c r="F372" t="n">
         <v>10077700</v>
@@ -7892,16 +7892,16 @@
         <v>44797</v>
       </c>
       <c r="B374" t="n">
-        <v>17.1483097076416</v>
+        <v>17.14830780029297</v>
       </c>
       <c r="C374" t="n">
-        <v>17.26391710340299</v>
+        <v>17.26391518319573</v>
       </c>
       <c r="D374" t="n">
-        <v>16.99416773830457</v>
+        <v>16.99416584810063</v>
       </c>
       <c r="E374" t="n">
-        <v>17.1483097076416</v>
+        <v>17.14830780029297</v>
       </c>
       <c r="F374" t="n">
         <v>5807100</v>
@@ -8052,16 +8052,16 @@
         <v>44809</v>
       </c>
       <c r="B382" t="n">
-        <v>18.73790168762207</v>
+        <v>18.7379035949707</v>
       </c>
       <c r="C382" t="n">
-        <v>18.91131002438889</v>
+        <v>18.91131194938891</v>
       </c>
       <c r="D382" t="n">
-        <v>18.12133197488807</v>
+        <v>18.12133381947549</v>
       </c>
       <c r="E382" t="n">
-        <v>18.39108133905402</v>
+        <v>18.39108321109948</v>
       </c>
       <c r="F382" t="n">
         <v>11861400</v>
@@ -8072,16 +8072,16 @@
         <v>44810</v>
       </c>
       <c r="B383" t="n">
-        <v>18.75716972351074</v>
+        <v>18.75716781616211</v>
       </c>
       <c r="C383" t="n">
-        <v>18.83424071476615</v>
+        <v>18.83423879958045</v>
       </c>
       <c r="D383" t="n">
-        <v>18.33328019036468</v>
+        <v>18.33327832611984</v>
       </c>
       <c r="E383" t="n">
-        <v>18.68973283585193</v>
+        <v>18.68973093536071</v>
       </c>
       <c r="F383" t="n">
         <v>7863100</v>
@@ -8112,16 +8112,16 @@
         <v>44813</v>
       </c>
       <c r="B385" t="n">
-        <v>18.15986824035645</v>
+        <v>18.15987014770508</v>
       </c>
       <c r="C385" t="n">
-        <v>18.62229414306423</v>
+        <v>18.6222960989819</v>
       </c>
       <c r="D385" t="n">
-        <v>18.08279725657182</v>
+        <v>18.08279915582561</v>
       </c>
       <c r="E385" t="n">
-        <v>18.47778627815769</v>
+        <v>18.47778821889757</v>
       </c>
       <c r="F385" t="n">
         <v>8752700</v>
@@ -8132,16 +8132,16 @@
         <v>44816</v>
       </c>
       <c r="B386" t="n">
-        <v>17.78414535522461</v>
+        <v>17.78414726257324</v>
       </c>
       <c r="C386" t="n">
-        <v>18.38144684992308</v>
+        <v>18.38144882133227</v>
       </c>
       <c r="D386" t="n">
-        <v>17.7070743724426</v>
+        <v>17.70707627152537</v>
       </c>
       <c r="E386" t="n">
-        <v>18.25620719197125</v>
+        <v>18.25620914994849</v>
       </c>
       <c r="F386" t="n">
         <v>10149200</v>
@@ -8172,16 +8172,16 @@
         <v>44818</v>
       </c>
       <c r="B388" t="n">
-        <v>17.70707511901855</v>
+        <v>17.70707321166992</v>
       </c>
       <c r="C388" t="n">
-        <v>17.8708511940252</v>
+        <v>17.87084926903514</v>
       </c>
       <c r="D388" t="n">
-        <v>17.36989070357892</v>
+        <v>17.3698888325507</v>
       </c>
       <c r="E388" t="n">
-        <v>17.44696168961044</v>
+        <v>17.44695981028038</v>
       </c>
       <c r="F388" t="n">
         <v>7347400</v>
@@ -8192,16 +8192,16 @@
         <v>44819</v>
       </c>
       <c r="B389" t="n">
-        <v>17.62036895751953</v>
+        <v>17.62037086486816</v>
       </c>
       <c r="C389" t="n">
-        <v>17.8419477760763</v>
+        <v>17.84194970741013</v>
       </c>
       <c r="D389" t="n">
-        <v>17.48549337610141</v>
+        <v>17.4854952688502</v>
       </c>
       <c r="E389" t="n">
-        <v>17.69743993082262</v>
+        <v>17.69744184651394</v>
       </c>
       <c r="F389" t="n">
         <v>7203900</v>
@@ -8212,16 +8212,16 @@
         <v>44820</v>
       </c>
       <c r="B390" t="n">
-        <v>17.24464797973633</v>
+        <v>17.24464988708496</v>
       </c>
       <c r="C390" t="n">
-        <v>17.62037061781912</v>
+        <v>17.62037256672464</v>
       </c>
       <c r="D390" t="n">
-        <v>17.06160371182508</v>
+        <v>17.06160559892805</v>
       </c>
       <c r="E390" t="n">
-        <v>17.49512912595248</v>
+        <v>17.49513106100564</v>
       </c>
       <c r="F390" t="n">
         <v>10140200</v>
@@ -8232,16 +8232,16 @@
         <v>44823</v>
       </c>
       <c r="B391" t="n">
-        <v>17.46623039245605</v>
+        <v>17.46622848510742</v>
       </c>
       <c r="C391" t="n">
-        <v>17.58183780571365</v>
+        <v>17.58183588574045</v>
       </c>
       <c r="D391" t="n">
-        <v>17.14831230289454</v>
+        <v>17.14831043026322</v>
       </c>
       <c r="E391" t="n">
-        <v>17.14831230289454</v>
+        <v>17.14831043026322</v>
       </c>
       <c r="F391" t="n">
         <v>7719100</v>
@@ -8292,16 +8292,16 @@
         <v>44826</v>
       </c>
       <c r="B394" t="n">
-        <v>17.36025619506836</v>
+        <v>17.36025810241699</v>
       </c>
       <c r="C394" t="n">
-        <v>17.88048487924835</v>
+        <v>17.88048684375383</v>
       </c>
       <c r="D394" t="n">
-        <v>16.94599896575775</v>
+        <v>16.94600082759248</v>
       </c>
       <c r="E394" t="n">
-        <v>17.66854013199238</v>
+        <v>17.66854207321177</v>
       </c>
       <c r="F394" t="n">
         <v>12903600</v>
@@ -8312,16 +8312,16 @@
         <v>44827</v>
       </c>
       <c r="B395" t="n">
-        <v>17.13867568969727</v>
+        <v>17.1386775970459</v>
       </c>
       <c r="C395" t="n">
-        <v>17.42769139326868</v>
+        <v>17.42769333278163</v>
       </c>
       <c r="D395" t="n">
-        <v>16.9652655325476</v>
+        <v>16.96526742059757</v>
       </c>
       <c r="E395" t="n">
-        <v>17.10977338433331</v>
+        <v>17.10977528846543</v>
       </c>
       <c r="F395" t="n">
         <v>12048200</v>
@@ -8352,16 +8352,16 @@
         <v>44831</v>
       </c>
       <c r="B397" t="n">
-        <v>17.12904167175293</v>
+        <v>17.12904357910156</v>
       </c>
       <c r="C397" t="n">
-        <v>17.49512835390313</v>
+        <v>17.49513030201615</v>
       </c>
       <c r="D397" t="n">
-        <v>16.86892643475522</v>
+        <v>16.86892831313957</v>
       </c>
       <c r="E397" t="n">
-        <v>17.2542813205757</v>
+        <v>17.25428324186998</v>
       </c>
       <c r="F397" t="n">
         <v>9260100</v>
@@ -8452,16 +8452,16 @@
         <v>44838</v>
       </c>
       <c r="B402" t="n">
-        <v>17.41806030273438</v>
+        <v>17.41805839538574</v>
       </c>
       <c r="C402" t="n">
-        <v>18.07316463743626</v>
+        <v>18.07316265835103</v>
       </c>
       <c r="D402" t="n">
-        <v>17.33135520916987</v>
+        <v>17.3313533113158</v>
       </c>
       <c r="E402" t="n">
-        <v>17.98645954387175</v>
+        <v>17.98645757428108</v>
       </c>
       <c r="F402" t="n">
         <v>18594600</v>
@@ -8492,16 +8492,16 @@
         <v>44840</v>
       </c>
       <c r="B404" t="n">
-        <v>17.44696235656738</v>
+        <v>17.44696426391602</v>
       </c>
       <c r="C404" t="n">
-        <v>17.63963891025314</v>
+        <v>17.6396408386657</v>
       </c>
       <c r="D404" t="n">
-        <v>17.30245264440641</v>
+        <v>17.30245453595685</v>
       </c>
       <c r="E404" t="n">
-        <v>17.63000480694126</v>
+        <v>17.63000673430058</v>
       </c>
       <c r="F404" t="n">
         <v>6691000</v>
@@ -8512,16 +8512,16 @@
         <v>44841</v>
       </c>
       <c r="B405" t="n">
-        <v>17.49513053894043</v>
+        <v>17.4951286315918</v>
       </c>
       <c r="C405" t="n">
-        <v>17.68780892467357</v>
+        <v>17.68780699631881</v>
       </c>
       <c r="D405" t="n">
-        <v>17.32172035928406</v>
+        <v>17.3217184708409</v>
       </c>
       <c r="E405" t="n">
-        <v>17.44696186126578</v>
+        <v>17.44695995916858</v>
       </c>
       <c r="F405" t="n">
         <v>11897600</v>
@@ -8552,16 +8552,16 @@
         <v>44845</v>
       </c>
       <c r="B407" t="n">
-        <v>18.32364463806152</v>
+        <v>18.32364654541016</v>
       </c>
       <c r="C407" t="n">
-        <v>18.59339216736995</v>
+        <v>18.5933941027972</v>
       </c>
       <c r="D407" t="n">
-        <v>17.85158462425454</v>
+        <v>17.8515864824654</v>
       </c>
       <c r="E407" t="n">
-        <v>18.15023446206769</v>
+        <v>18.15023635136567</v>
       </c>
       <c r="F407" t="n">
         <v>12287200</v>
@@ -8572,16 +8572,16 @@
         <v>44847</v>
       </c>
       <c r="B408" t="n">
-        <v>18.75716972351074</v>
+        <v>18.75716781616211</v>
       </c>
       <c r="C408" t="n">
-        <v>18.99801680087357</v>
+        <v>18.99801486903407</v>
       </c>
       <c r="D408" t="n">
-        <v>17.93829113049103</v>
+        <v>17.93828930641119</v>
       </c>
       <c r="E408" t="n">
-        <v>18.17913820785386</v>
+        <v>18.17913635928316</v>
       </c>
       <c r="F408" t="n">
         <v>20665700</v>
@@ -8652,16 +8652,16 @@
         <v>44853</v>
       </c>
       <c r="B412" t="n">
-        <v>17.67817306518555</v>
+        <v>17.67817497253418</v>
       </c>
       <c r="C412" t="n">
-        <v>17.97682287963343</v>
+        <v>17.97682481920425</v>
       </c>
       <c r="D412" t="n">
-        <v>17.28318406744306</v>
+        <v>17.2831859321752</v>
       </c>
       <c r="E412" t="n">
-        <v>17.47586059651518</v>
+        <v>17.47586248203574</v>
       </c>
       <c r="F412" t="n">
         <v>27062400</v>
@@ -8712,16 +8712,16 @@
         <v>44858</v>
       </c>
       <c r="B415" t="n">
-        <v>18.0057258605957</v>
+        <v>18.00572776794434</v>
       </c>
       <c r="C415" t="n">
-        <v>18.36217846337067</v>
+        <v>18.36218040847837</v>
       </c>
       <c r="D415" t="n">
-        <v>17.54329813095674</v>
+        <v>17.54329998932035</v>
       </c>
       <c r="E415" t="n">
-        <v>17.91902077613322</v>
+        <v>17.91902267429717</v>
       </c>
       <c r="F415" t="n">
         <v>16227000</v>
@@ -8812,16 +8812,16 @@
         <v>44865</v>
       </c>
       <c r="B420" t="n">
-        <v>19.09435653686523</v>
+        <v>19.0943546295166</v>
       </c>
       <c r="C420" t="n">
-        <v>19.24849852371545</v>
+        <v>19.24849660096946</v>
       </c>
       <c r="D420" t="n">
-        <v>18.13096820029268</v>
+        <v>18.13096638917758</v>
       </c>
       <c r="E420" t="n">
-        <v>18.29474429101071</v>
+        <v>18.2947424635359</v>
       </c>
       <c r="F420" t="n">
         <v>18379300</v>
@@ -8832,16 +8832,16 @@
         <v>44866</v>
       </c>
       <c r="B421" t="n">
-        <v>19.16179084777832</v>
+        <v>19.16178894042969</v>
       </c>
       <c r="C421" t="n">
-        <v>19.48934298513498</v>
+        <v>19.48934104518208</v>
       </c>
       <c r="D421" t="n">
-        <v>18.67046264174334</v>
+        <v>18.67046078330111</v>
       </c>
       <c r="E421" t="n">
-        <v>18.88240922327834</v>
+        <v>18.88240734373912</v>
       </c>
       <c r="F421" t="n">
         <v>15316600</v>
@@ -8852,16 +8852,16 @@
         <v>44868</v>
       </c>
       <c r="B422" t="n">
-        <v>19.62421798706055</v>
+        <v>19.62421989440918</v>
       </c>
       <c r="C422" t="n">
-        <v>19.74945764164638</v>
+        <v>19.74945956116751</v>
       </c>
       <c r="D422" t="n">
-        <v>18.69936438101601</v>
+        <v>18.69936619847478</v>
       </c>
       <c r="E422" t="n">
-        <v>18.69936438101601</v>
+        <v>18.69936619847478</v>
       </c>
       <c r="F422" t="n">
         <v>9732300</v>
@@ -8872,16 +8872,16 @@
         <v>44869</v>
       </c>
       <c r="B423" t="n">
-        <v>19.79762840270996</v>
+        <v>19.79763031005859</v>
       </c>
       <c r="C423" t="n">
-        <v>19.98067269026426</v>
+        <v>19.9806746152478</v>
       </c>
       <c r="D423" t="n">
-        <v>19.60495184937882</v>
+        <v>19.60495373816456</v>
       </c>
       <c r="E423" t="n">
-        <v>19.81689660929827</v>
+        <v>19.81689851850324</v>
       </c>
       <c r="F423" t="n">
         <v>15655600</v>
@@ -8912,16 +8912,16 @@
         <v>44873</v>
       </c>
       <c r="B425" t="n">
-        <v>19.22922897338867</v>
+        <v>19.2292308807373</v>
       </c>
       <c r="C425" t="n">
-        <v>19.45080967184277</v>
+        <v>19.45081160117001</v>
       </c>
       <c r="D425" t="n">
-        <v>19.0750869973007</v>
+        <v>19.07508888935998</v>
       </c>
       <c r="E425" t="n">
-        <v>19.26776538616931</v>
+        <v>19.26776729734038</v>
       </c>
       <c r="F425" t="n">
         <v>10214300</v>
@@ -8932,16 +8932,16 @@
         <v>44874</v>
       </c>
       <c r="B426" t="n">
-        <v>19.65312004089355</v>
+        <v>19.65311813354492</v>
       </c>
       <c r="C426" t="n">
-        <v>20.09627959384678</v>
+        <v>20.09627764348921</v>
       </c>
       <c r="D426" t="n">
-        <v>19.1328913385332</v>
+        <v>19.13288948167312</v>
       </c>
       <c r="E426" t="n">
-        <v>19.1328913385332</v>
+        <v>19.13288948167312</v>
       </c>
       <c r="F426" t="n">
         <v>19633400</v>
@@ -8952,16 +8952,16 @@
         <v>44875</v>
       </c>
       <c r="B427" t="n">
-        <v>18.80533790588379</v>
+        <v>18.80533981323242</v>
       </c>
       <c r="C427" t="n">
-        <v>19.64348460199946</v>
+        <v>19.64348659435789</v>
       </c>
       <c r="D427" t="n">
-        <v>18.43924936475051</v>
+        <v>18.43925123496827</v>
       </c>
       <c r="E427" t="n">
-        <v>19.64348460199946</v>
+        <v>19.64348659435789</v>
       </c>
       <c r="F427" t="n">
         <v>13893700</v>
@@ -9032,16 +9032,16 @@
         <v>44882</v>
       </c>
       <c r="B431" t="n">
-        <v>18.78607177734375</v>
+        <v>18.78606986999512</v>
       </c>
       <c r="C431" t="n">
-        <v>18.90167918140427</v>
+        <v>18.90167726231802</v>
       </c>
       <c r="D431" t="n">
-        <v>18.0538964516734</v>
+        <v>18.05389461866248</v>
       </c>
       <c r="E431" t="n">
-        <v>18.66083210733576</v>
+        <v>18.6608302127027</v>
       </c>
       <c r="F431" t="n">
         <v>10826800</v>
@@ -9052,16 +9052,16 @@
         <v>44883</v>
       </c>
       <c r="B432" t="n">
-        <v>18.44888687133789</v>
+        <v>18.44888496398926</v>
       </c>
       <c r="C432" t="n">
-        <v>19.0269202593795</v>
+        <v>19.02691829227056</v>
       </c>
       <c r="D432" t="n">
-        <v>18.44888687133789</v>
+        <v>18.44888496398926</v>
       </c>
       <c r="E432" t="n">
-        <v>18.78607316748862</v>
+        <v>18.78607122527979</v>
       </c>
       <c r="F432" t="n">
         <v>9969800</v>
@@ -9072,16 +9072,16 @@
         <v>44886</v>
       </c>
       <c r="B433" t="n">
-        <v>18.98838043212891</v>
+        <v>18.98838233947754</v>
       </c>
       <c r="C433" t="n">
-        <v>19.02691684191824</v>
+        <v>19.02691875313779</v>
       </c>
       <c r="D433" t="n">
-        <v>18.58375915444382</v>
+        <v>18.58376102114898</v>
       </c>
       <c r="E433" t="n">
-        <v>18.60302552182134</v>
+        <v>18.60302739046176</v>
       </c>
       <c r="F433" t="n">
         <v>10461100</v>
@@ -9092,16 +9092,16 @@
         <v>44887</v>
       </c>
       <c r="B434" t="n">
-        <v>18.75716972351074</v>
+        <v>18.75716781616211</v>
       </c>
       <c r="C434" t="n">
-        <v>19.39300586074722</v>
+        <v>19.39300388874271</v>
       </c>
       <c r="D434" t="n">
-        <v>18.62229594819312</v>
+        <v>18.62229405455931</v>
       </c>
       <c r="E434" t="n">
-        <v>19.07508779212898</v>
+        <v>19.07508585245241</v>
       </c>
       <c r="F434" t="n">
         <v>9653000</v>
@@ -9252,16 +9252,16 @@
         <v>44897</v>
       </c>
       <c r="B442" t="n">
-        <v>19.78799438476562</v>
+        <v>19.78799629211426</v>
       </c>
       <c r="C442" t="n">
-        <v>19.97103681859475</v>
+        <v>19.97103874358669</v>
       </c>
       <c r="D442" t="n">
-        <v>19.01728272713333</v>
+        <v>19.01728456019369</v>
       </c>
       <c r="E442" t="n">
-        <v>19.11362191402701</v>
+        <v>19.11362375637343</v>
       </c>
       <c r="F442" t="n">
         <v>24428900</v>
@@ -9292,16 +9292,16 @@
         <v>44901</v>
       </c>
       <c r="B444" t="n">
-        <v>19.22922897338867</v>
+        <v>19.2292308807373</v>
       </c>
       <c r="C444" t="n">
-        <v>19.81689640567237</v>
+        <v>19.81689837131178</v>
       </c>
       <c r="D444" t="n">
-        <v>18.97874964038369</v>
+        <v>18.97875152288726</v>
       </c>
       <c r="E444" t="n">
-        <v>19.74945952082355</v>
+        <v>19.74946147977388</v>
       </c>
       <c r="F444" t="n">
         <v>9745600</v>
@@ -9312,16 +9312,16 @@
         <v>44902</v>
       </c>
       <c r="B445" t="n">
-        <v>19.36410522460938</v>
+        <v>19.36410331726074</v>
       </c>
       <c r="C445" t="n">
-        <v>19.48934489527705</v>
+        <v>19.48934297559241</v>
       </c>
       <c r="D445" t="n">
-        <v>18.82460829035904</v>
+        <v>18.82460643615043</v>
       </c>
       <c r="E445" t="n">
-        <v>19.17142682933272</v>
+        <v>19.17142494096275</v>
       </c>
       <c r="F445" t="n">
         <v>7439200</v>
@@ -9352,16 +9352,16 @@
         <v>44904</v>
       </c>
       <c r="B447" t="n">
-        <v>18.57412528991699</v>
+        <v>18.57412719726562</v>
       </c>
       <c r="C447" t="n">
-        <v>18.7571677262095</v>
+        <v>18.75716965235448</v>
       </c>
       <c r="D447" t="n">
-        <v>18.25620725515131</v>
+        <v>18.25620912985342</v>
       </c>
       <c r="E447" t="n">
-        <v>18.57412528991699</v>
+        <v>18.57412719726562</v>
       </c>
       <c r="F447" t="n">
         <v>14833900</v>
@@ -9372,16 +9372,16 @@
         <v>44907</v>
       </c>
       <c r="B448" t="n">
-        <v>18.2562084197998</v>
+        <v>18.25621032714844</v>
       </c>
       <c r="C448" t="n">
-        <v>18.6704638316658</v>
+        <v>18.67046578229448</v>
       </c>
       <c r="D448" t="n">
-        <v>17.87085164245525</v>
+        <v>17.87085350954307</v>
       </c>
       <c r="E448" t="n">
-        <v>18.45851907414013</v>
+        <v>18.45852100262552</v>
       </c>
       <c r="F448" t="n">
         <v>10851800</v>
@@ -9392,16 +9392,16 @@
         <v>44908</v>
       </c>
       <c r="B449" t="n">
-        <v>17.94792175292969</v>
+        <v>17.94792366027832</v>
       </c>
       <c r="C449" t="n">
-        <v>18.52595505316863</v>
+        <v>18.5259570219456</v>
       </c>
       <c r="D449" t="n">
-        <v>17.89975307687528</v>
+        <v>17.89975497910497</v>
       </c>
       <c r="E449" t="n">
-        <v>18.52595505316863</v>
+        <v>18.5259570219456</v>
       </c>
       <c r="F449" t="n">
         <v>13648600</v>
@@ -9432,16 +9432,16 @@
         <v>44910</v>
       </c>
       <c r="B451" t="n">
-        <v>18.41998481750488</v>
+        <v>18.41998672485352</v>
       </c>
       <c r="C451" t="n">
-        <v>18.75716924723731</v>
+        <v>18.75717118950064</v>
       </c>
       <c r="D451" t="n">
-        <v>18.0924326536071</v>
+        <v>18.09243452703844</v>
       </c>
       <c r="E451" t="n">
-        <v>18.11169902279372</v>
+        <v>18.11170089822004</v>
       </c>
       <c r="F451" t="n">
         <v>15735500</v>
@@ -9512,16 +9512,16 @@
         <v>44916</v>
       </c>
       <c r="B455" t="n">
-        <v>19.44117546081543</v>
+        <v>19.4411735534668</v>
       </c>
       <c r="C455" t="n">
-        <v>19.67238842366494</v>
+        <v>19.6723864936323</v>
       </c>
       <c r="D455" t="n">
-        <v>19.07508689149907</v>
+        <v>19.07508502006691</v>
       </c>
       <c r="E455" t="n">
-        <v>19.30630169186587</v>
+        <v>19.30629979774953</v>
       </c>
       <c r="F455" t="n">
         <v>13319200</v>
@@ -9532,16 +9532,16 @@
         <v>44917</v>
       </c>
       <c r="B456" t="n">
-        <v>19.38337326049805</v>
+        <v>19.38337516784668</v>
       </c>
       <c r="C456" t="n">
-        <v>19.52788113692095</v>
+        <v>19.52788305848934</v>
       </c>
       <c r="D456" t="n">
-        <v>19.07508746327389</v>
+        <v>19.07508934028681</v>
       </c>
       <c r="E456" t="n">
-        <v>19.52788113692095</v>
+        <v>19.52788305848934</v>
       </c>
       <c r="F456" t="n">
         <v>7183700</v>
@@ -9572,16 +9572,16 @@
         <v>44921</v>
       </c>
       <c r="B458" t="n">
-        <v>19.20033073425293</v>
+        <v>19.2003288269043</v>
       </c>
       <c r="C458" t="n">
-        <v>19.32557041532036</v>
+        <v>19.3255684955305</v>
       </c>
       <c r="D458" t="n">
-        <v>18.84387622464675</v>
+        <v>18.84387435270808</v>
       </c>
       <c r="E458" t="n">
-        <v>19.07508921566799</v>
+        <v>19.07508732076077</v>
       </c>
       <c r="F458" t="n">
         <v>2369600</v>
@@ -9612,16 +9612,16 @@
         <v>44923</v>
       </c>
       <c r="B460" t="n">
-        <v>18.71863555908203</v>
+        <v>18.7186336517334</v>
       </c>
       <c r="C460" t="n">
-        <v>18.94984853794273</v>
+        <v>18.94984660703449</v>
       </c>
       <c r="D460" t="n">
-        <v>18.26584186765209</v>
+        <v>18.26584000644119</v>
       </c>
       <c r="E460" t="n">
-        <v>18.68973324765541</v>
+        <v>18.6897313432518</v>
       </c>
       <c r="F460" t="n">
         <v>8329700</v>
@@ -28752,19 +28752,39 @@
         <v>46324</v>
       </c>
       <c r="B1417" t="n">
-        <v>7.81</v>
+        <v>7.809999942779541</v>
       </c>
       <c r="C1417" t="n">
-        <v>8.050000000000001</v>
+        <v>8.050000190734863</v>
       </c>
       <c r="D1417" t="n">
-        <v>7.68</v>
+        <v>7.679999828338623</v>
       </c>
       <c r="E1417" t="n">
-        <v>7.88</v>
+        <v>7.880000114440918</v>
       </c>
       <c r="F1417" t="n">
         <v>24884400</v>
+      </c>
+    </row>
+    <row r="1418">
+      <c r="A1418" s="1" t="n">
+        <v>46325</v>
+      </c>
+      <c r="B1418" t="n">
+        <v>7.88</v>
+      </c>
+      <c r="C1418" t="n">
+        <v>8.029999999999999</v>
+      </c>
+      <c r="D1418" t="n">
+        <v>7.62</v>
+      </c>
+      <c r="E1418" t="n">
+        <v>7.8</v>
+      </c>
+      <c r="F1418" t="n">
+        <v>28592300</v>
       </c>
     </row>
   </sheetData>

</xml_diff>